<commit_message>
Planilha de manutenção preventiva
</commit_message>
<xml_diff>
--- a/ordens_de_servico.xlsx
+++ b/ordens_de_servico.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WIKI\Documents\Fabrício\Projetos\excel-data-analysis\1. controle-de-manutenção-preventiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEE51F5-5BF2-48AF-B53B-A81D9E340B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF10C45-22C1-4173-B2B8-8357C0EDB219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{90E3A9FA-0E00-48D2-BFE9-7577E25EE9AC}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1023" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="171">
   <si>
     <t>ID_OS</t>
   </si>
@@ -524,9 +524,6 @@
     <t>Responsável</t>
   </si>
   <si>
-    <t>Em andameto</t>
-  </si>
-  <si>
     <t>STATUS DAS OS POR RESPONSÁVEL</t>
   </si>
   <si>
@@ -534,6 +531,12 @@
   </si>
   <si>
     <t>Desvio_de_Prazo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usei a validação de dados para filtrar os responsaveis. Usei o CONT.SES para trazer os valores das OS, abertas, em andamento e concluída. Usei o SE com O DATADIF como condição para me dar em dias as OS que foram concluídas, quantos dias antes eram foram concluídas, se foram concluídas no prazo era igual a zero e se a data de conclusão foi feita depois do prazo, os dias seriam negativos e na cor vermelha. usei a condição SE para me indicar o status da atividade, baseada no responsavel que será filtrado na validação de dados. Usei a fórmula HOJE no título da planilha, assim que for salvo ficará com a data que foi salvo. </t>
+  </si>
+  <si>
+    <t>Geral</t>
   </si>
 </sst>
 </file>
@@ -1225,7 +1228,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1292,16 +1295,19 @@
     <xf numFmtId="0" fontId="13" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1947,6 +1953,7 @@
                 <a:ea typeface="Calibri"/>
                 <a:cs typeface="Calibri"/>
               </a:rPr>
+              <a:pPr/>
               <a:t>09/10/2026</a:t>
             </a:fld>
             <a:endParaRPr lang="pt-BR" sz="1100" b="0" i="1">
@@ -5768,10 +5775,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:42" s="17" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H3" s="28"/>
+      <c r="H3" s="26"/>
       <c r="I3" s="18"/>
       <c r="J3" s="18"/>
-      <c r="AP3" s="29">
+      <c r="AP3" s="27">
         <f ca="1">TODAY()</f>
         <v>46304</v>
       </c>
@@ -5782,16 +5789,16 @@
         <v>165</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>21</v>
+        <v>170</v>
       </c>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="D11" s="27"/>
+      <c r="C11" s="28" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="29"/>
       <c r="E11" s="1"/>
       <c r="F11" s="19" t="s">
         <v>0</v>
@@ -5803,7 +5810,7 @@
         <v>6</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J11" s="25" t="s">
         <v>7</v>
@@ -5814,8 +5821,8 @@
         <v>91</v>
       </c>
       <c r="D12" s="21">
-        <f>COUNTIFS(ordens_de_servico!J:J,resumo!$D$9,ordens_de_servico!I:I,"Aberta")</f>
-        <v>7</v>
+        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C12),COUNTIFS(ordens_de_servico!J:J,resumo!D9,ordens_de_servico!I:I,resumo!C12))</f>
+        <v>45</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="7" t="s">
@@ -5838,11 +5845,11 @@
     </row>
     <row r="13" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="20" t="s">
-        <v>166</v>
+        <v>76</v>
       </c>
       <c r="D13" s="21">
-        <f>COUNTIFS(ordens_de_servico!J:J,resumo!$D$9,ordens_de_servico!I:I,"Em andamento")</f>
-        <v>3</v>
+        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C13),COUNTIFS(ordens_de_servico!J:J,resumo!D10,ordens_de_servico!I:I,resumo!C13))</f>
+        <v>21</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="7" t="s">
@@ -5860,7 +5867,7 @@
       </c>
       <c r="J13" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J3,ordens_de_servico!I3,"")</f>
-        <v>Concluída</v>
+        <v/>
       </c>
     </row>
     <row r="14" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5868,8 +5875,8 @@
         <v>14</v>
       </c>
       <c r="D14" s="21">
-        <f>COUNTIFS(ordens_de_servico!J:J,resumo!$D$9,ordens_de_servico!I:I,"Concluída")</f>
-        <v>5</v>
+        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C14),COUNTIFS(ordens_de_servico!J:J,resumo!D11,ordens_de_servico!I:I,resumo!C14))</f>
+        <v>34</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="7" t="s">
@@ -5892,11 +5899,11 @@
     </row>
     <row r="15" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C15" s="22" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D15" s="23">
         <f>SUM(D12:D14)</f>
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="E15" s="6"/>
       <c r="F15" s="7" t="s">
@@ -5959,6 +5966,9 @@
     </row>
     <row r="18" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C18" s="1"/>
+      <c r="D18" t="s">
+        <v>169</v>
+      </c>
       <c r="F18" s="7" t="s">
         <v>35</v>
       </c>
@@ -5978,7 +5988,7 @@
       </c>
     </row>
     <row r="19" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="1"/>
+      <c r="C19" s="30"/>
       <c r="F19" s="7" t="s">
         <v>38</v>
       </c>
@@ -5994,7 +6004,7 @@
       </c>
       <c r="J19" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J9,ordens_de_servico!I9,"")</f>
-        <v>Concluída</v>
+        <v/>
       </c>
     </row>
     <row r="20" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6206,7 +6216,7 @@
       </c>
       <c r="J30" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J20,ordens_de_servico!I20,"")</f>
-        <v>Concluída</v>
+        <v/>
       </c>
     </row>
     <row r="31" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6282,7 +6292,7 @@
       </c>
       <c r="J34" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J24,ordens_de_servico!I24,"")</f>
-        <v>Concluída</v>
+        <v/>
       </c>
     </row>
     <row r="35" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6510,7 +6520,7 @@
       </c>
       <c r="J46" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J36,ordens_de_servico!I36,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="47" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6624,7 +6634,7 @@
       </c>
       <c r="J52" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J42,ordens_de_servico!I42,"")</f>
-        <v>Concluída</v>
+        <v/>
       </c>
     </row>
     <row r="53" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6662,7 +6672,7 @@
       </c>
       <c r="J54" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J44,ordens_de_servico!I44,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="55" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6871,7 +6881,7 @@
       </c>
       <c r="J65" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J55,ordens_de_servico!I55,"")</f>
-        <v>Em andamento</v>
+        <v/>
       </c>
     </row>
     <row r="66" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7023,7 +7033,7 @@
       </c>
       <c r="J73" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J63,ordens_de_servico!I63,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="74" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7080,7 +7090,7 @@
       </c>
       <c r="J76" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J66,ordens_de_servico!I66,"")</f>
-        <v>Em andamento</v>
+        <v/>
       </c>
     </row>
     <row r="77" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7251,7 +7261,7 @@
       </c>
       <c r="J85" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J75,ordens_de_servico!I75,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="86" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7327,7 +7337,7 @@
       </c>
       <c r="J89" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J79,ordens_de_servico!I79,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="90" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7365,7 +7375,7 @@
       </c>
       <c r="J91" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J81,ordens_de_servico!I81,"")</f>
-        <v>Em andamento</v>
+        <v/>
       </c>
     </row>
     <row r="92" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7479,7 +7489,7 @@
       </c>
       <c r="J97" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J87,ordens_de_servico!I87,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="98" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7669,7 +7679,7 @@
       </c>
       <c r="J107" s="11" t="str">
         <f>IF($D$9=ordens_de_servico!J97,ordens_de_servico!I97,"")</f>
-        <v>Aberta</v>
+        <v/>
       </c>
     </row>
     <row r="108" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7774,7 +7784,7 @@
   </conditionalFormatting>
   <dataValidations xWindow="472" yWindow="308" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor não permitido" error="Escolha uma das opções da lista. Não é possível digitar outro texto neste campo." promptTitle="Filtro" prompt="Selecione o responsável desejado" sqref="D9" xr:uid="{78BEE481-69E3-40B6-91E7-F4B089E9070C}">
-      <formula1>"Ana Souza, Carlos Lima, Juliana Alves, Marcos Pereira, Paula Mendes, Rafael Costa"</formula1>
+      <formula1>"Geral,Ana Souza, Carlos Lima, Juliana Alves, Marcos Pereira, Paula Mendes, Rafael Costa"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Controle de manutenção preventiva
</commit_message>
<xml_diff>
--- a/ordens_de_servico.xlsx
+++ b/ordens_de_servico.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WIKI\Documents\Fabrício\Projetos\excel-data-analysis\1. controle-de-manutenção-preventiva\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF10C45-22C1-4173-B2B8-8357C0EDB219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C009954C-1D80-4947-B2BA-BCD21A861528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{90E3A9FA-0E00-48D2-BFE9-7577E25EE9AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="2" xr2:uid="{90E3A9FA-0E00-48D2-BFE9-7577E25EE9AC}"/>
   </bookViews>
   <sheets>
-    <sheet name="ordens_de_servico" sheetId="1" r:id="rId1"/>
-    <sheet name="resumo" sheetId="3" r:id="rId2"/>
+    <sheet name="csv" sheetId="4" r:id="rId1"/>
+    <sheet name="ordens_de_servico" sheetId="1" r:id="rId2"/>
+    <sheet name="resumo" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">resumo!$F$11:$J$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">resumo!$F$7:$J$107</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="271">
   <si>
     <t>ID_OS</t>
   </si>
@@ -524,19 +525,319 @@
     <t>Responsável</t>
   </si>
   <si>
-    <t>STATUS DAS OS POR RESPONSÁVEL</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
     <t>Desvio_de_Prazo</t>
   </si>
   <si>
-    <t xml:space="preserve">Usei a validação de dados para filtrar os responsaveis. Usei o CONT.SES para trazer os valores das OS, abertas, em andamento e concluída. Usei o SE com O DATADIF como condição para me dar em dias as OS que foram concluídas, quantos dias antes eram foram concluídas, se foram concluídas no prazo era igual a zero e se a data de conclusão foi feita depois do prazo, os dias seriam negativos e na cor vermelha. usei a condição SE para me indicar o status da atividade, baseada no responsavel que será filtrado na validação de dados. Usei a fórmula HOJE no título da planilha, assim que for salvo ficará com a data que foi salvo. </t>
-  </si>
-  <si>
     <t>Geral</t>
+  </si>
+  <si>
+    <t>ID_OS;TAG;Equipamento;Setor;Tipo;Data_Abertura;Prazo;Data_Conclusao;Status;Responsavel;Prioridade</t>
+  </si>
+  <si>
+    <t>OS-001;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-07-22;2026-08-21;2026-08-27;Concluída;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-002;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-07-22;2026-08-21;2026-08-19;Concluída;Rafael Costa;Média</t>
+  </si>
+  <si>
+    <t>OS-003;TRN-001;Torno CNC;Produção;Preventiva;2026-07-24;2026-08-23;2026-08-18;Concluída;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-004;TRN-001;Torno CNC;Produção;Preventiva;2026-07-25;2026-08-14;2026-08-11;Concluída;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-005;BMB-002;Bomba centrífuga 2;Utilidades;Preventiva;2026-07-28;2026-08-12;2026-08-07;Concluída;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-006;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-08-05;2026-08-20;2026-08-20;Concluída;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-007;PRS-001;Prensa hidráulica;Produção;Preventiva;2026-08-05;2026-08-25;2026-08-20;Concluída;Paula Mendes;Alta</t>
+  </si>
+  <si>
+    <t>OS-008;GER-001;Gerador diesel;Elétrica;Preventiva;2026-08-06;2026-08-13;2026-08-11;Concluída;Rafael Costa;Baixa</t>
+  </si>
+  <si>
+    <t>OS-009;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-08-07;2026-08-17;2026-08-16;Concluída;Ana Souza;Baixa</t>
+  </si>
+  <si>
+    <t>OS-010;TRN-001;Torno CNC;Produção;Preventiva;2026-08-08;2026-08-15;2026-08-12;Concluída;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-011;QDF-002;Quadro de distribuição B;Elétrica;Preventiva;2026-08-08;2026-08-15;2026-08-21;Concluída;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-012;ELV-001;Elevador de carga;Predial;Preventiva;2026-08-10;2026-08-20;2026-08-18;Concluída;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-013;BMB-003;Bomba dosadora;Utilidades;Preventiva;2026-08-11;2026-08-31;2026-08-27;Concluída;Carlos Lima;Baixa</t>
+  </si>
+  <si>
+    <t>OS-014;TRN-001;Torno CNC;Produção;Preventiva;2026-08-12;2026-09-01;2026-08-28;Concluída;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-015;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-08-15;2026-08-22;2026-08-19;Concluída;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-016;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-08-16;2026-09-15;2026-09-15;Concluída;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-017;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-08-17;2026-09-01;2026-08-29;Concluída;Ana Souza;Baixa</t>
+  </si>
+  <si>
+    <t>OS-018;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-08-18;2026-08-28;2026-08-28;Concluída;Juliana Alves;Baixa</t>
+  </si>
+  <si>
+    <t>OS-019;BCI-001;Bomba de incêndio;Predial;Preventiva;2026-08-19;2026-09-08;2026-09-16;Concluída;Rafael Costa;Alta</t>
+  </si>
+  <si>
+    <t>OS-020;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-08-19;2026-08-26;2026-08-23;Concluída;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-021;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-08-20;2026-08-27;2026-09-05;Concluída;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-022;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-08-20;2026-09-09;;Em andamento;Paula Mendes;Baixa</t>
+  </si>
+  <si>
+    <t>OS-023;BCI-001;Bomba de incêndio;Predial;Preventiva;2026-08-22;2026-09-11;2026-09-13;Concluída;Rafael Costa;Baixa</t>
+  </si>
+  <si>
+    <t>OS-024;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-08-22;2026-09-11;2026-09-08;Concluída;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-025;ELV-002;Elevador social;Predial;Preventiva;2026-08-23;2026-09-02;2026-09-10;Concluída;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-026;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-08-24;2026-09-13;2026-09-17;Concluída;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-027;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-08-24;2026-09-23;2026-09-26;Concluída;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-028;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-08-28;2026-09-17;;Em andamento;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-029;QDF-002;Quadro de distribuição B;Elétrica;Preventiva;2026-08-28;2026-09-04;2026-09-10;Concluída;Paula Mendes;Baixa</t>
+  </si>
+  <si>
+    <t>OS-030;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-08-30;2026-09-06;;Em andamento;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-031;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-08-30;2026-09-19;2026-09-16;Concluída;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-032;BCI-001;Bomba de incêndio;Predial;Preventiva;2026-08-31;2026-09-07;;Em andamento;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-033;BMB-002;Bomba centrífuga 2;Utilidades;Preventiva;2026-08-31;2026-09-10;2026-09-18;Concluída;Paula Mendes;Baixa</t>
+  </si>
+  <si>
+    <t>OS-034;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-09-01;2026-09-11;;Aberta;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-035;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-09-01;2026-09-11;;Aberta;Rafael Costa;Alta</t>
+  </si>
+  <si>
+    <t>OS-036;TRN-001;Torno CNC;Produção;Preventiva;2026-09-02;2026-09-17;2026-09-17;Concluída;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-037;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-09-02;2026-09-22;;Aberta;Paula Mendes;Alta</t>
+  </si>
+  <si>
+    <t>OS-038;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-09-03;2026-09-23;2026-09-22;Concluída;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-039;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-09-08;2026-09-18;2026-09-21;Concluída;Juliana Alves;Alta</t>
+  </si>
+  <si>
+    <t>OS-040;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-09-08;2026-10-08;;Aberta;Paula Mendes;Baixa</t>
+  </si>
+  <si>
+    <t>OS-041;ESP-001;Esteira transportadora;Produção;Preventiva;2026-09-08;2026-09-18;2026-09-14;Concluída;Rafael Costa;Baixa</t>
+  </si>
+  <si>
+    <t>OS-042;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-09-08;2026-09-18;2026-09-24;Concluída;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-043;PRS-001;Prensa hidráulica;Produção;Preventiva;2026-09-09;2026-09-16;;Aberta;Rafael Costa;Média</t>
+  </si>
+  <si>
+    <t>OS-044;BCI-001;Bomba de incêndio;Predial;Preventiva;2026-09-09;2026-10-09;;Aberta;Juliana Alves;Baixa</t>
+  </si>
+  <si>
+    <t>OS-045;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-09-09;2026-10-09;;Aberta;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-046;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-09-09;2026-10-09;;Aberta;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-047;EXA-001;Exaustor industrial;Produção;Preventiva;2026-09-09;2026-10-09;;Em andamento;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-048;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-09-12;2026-10-02;;Em andamento;Ana Souza;Baixa</t>
+  </si>
+  <si>
+    <t>OS-049;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-09-14;2026-09-29;;Em andamento;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-050;GER-001;Gerador diesel;Elétrica;Preventiva;2026-09-15;2026-10-15;;Aberta;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-051;EXA-001;Exaustor industrial;Produção;Preventiva;2026-09-17;2026-09-24;;Aberta;Juliana Alves;Baixa</t>
+  </si>
+  <si>
+    <t>OS-052;PRS-001;Prensa hidráulica;Produção;Preventiva;2026-09-18;2026-10-08;;Em andamento;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-053;CMP-001;Compressor de ar 1;Utilidades;Preventiva;2026-09-21;2026-10-06;;Em andamento;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-054;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-09-22;2026-10-07;;Em andamento;Rafael Costa;Média</t>
+  </si>
+  <si>
+    <t>OS-055;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-09-24;2026-10-14;;Aberta;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-056;BMB-003;Bomba dosadora;Utilidades;Preventiva;2026-09-25;2026-10-05;;Aberta;Carlos Lima;Baixa</t>
+  </si>
+  <si>
+    <t>OS-057;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-09-25;2026-10-25;;Aberta;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-058;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-09-25;2026-10-15;;Aberta;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-059;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-09-26;2026-10-16;;Em andamento;Carlos Lima;Baixa</t>
+  </si>
+  <si>
+    <t>OS-060;EXA-001;Exaustor industrial;Produção;Preventiva;2026-09-26;2026-10-11;;Em andamento;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-061;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-09-26;2026-10-03;;Em andamento;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-062;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-09-26;2026-10-06;;Aberta;Rafael Costa;Baixa</t>
+  </si>
+  <si>
+    <t>OS-063;ESP-001;Esteira transportadora;Produção;Preventiva;2026-09-26;2026-10-16;;Aberta;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-064;EXA-001;Exaustor industrial;Produção;Preventiva;2026-09-26;2026-10-06;;Aberta;Juliana Alves;Baixa</t>
+  </si>
+  <si>
+    <t>OS-065;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-09-27;2026-10-27;;Em andamento;Rafael Costa;Baixa</t>
+  </si>
+  <si>
+    <t>OS-066;QDF-002;Quadro de distribuição B;Elétrica;Preventiva;2026-09-28;2026-10-05;;Aberta;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-067;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-09-28;2026-10-08;;Aberta;Marcos Pereira;Alta</t>
+  </si>
+  <si>
+    <t>OS-068;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-09-28;2026-10-05;;Em andamento;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-069;EXA-001;Exaustor industrial;Produção;Preventiva;2026-09-28;2026-10-18;;Aberta;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-070;ELV-002;Elevador social;Predial;Preventiva;2026-09-29;2026-10-29;;Aberta;Ana Souza;Baixa</t>
+  </si>
+  <si>
+    <t>OS-071;CMP-001;Compressor de ar 1;Utilidades;Preventiva;2026-09-29;2026-10-09;;Aberta;Marcos Pereira;Alta</t>
+  </si>
+  <si>
+    <t>OS-072;ESP-001;Esteira transportadora;Produção;Preventiva;2026-09-30;2026-10-15;;Em andamento;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-073;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-09-30;2026-10-10;;Aberta;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-074;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-10-02;2026-10-09;;Aberta;Rafael Costa;Alta</t>
+  </si>
+  <si>
+    <t>OS-075;BMB-003;Bomba dosadora;Utilidades;Preventiva;2026-10-03;2026-11-02;;Aberta;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-076;BMB-002;Bomba centrífuga 2;Utilidades;Preventiva;2026-10-04;2026-10-14;;Em andamento;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-077;QDF-002;Quadro de distribuição B;Elétrica;Preventiva;2026-10-05;2026-10-15;;Em andamento;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-078;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-10-07;2026-10-27;;Aberta;Rafael Costa;Alta</t>
+  </si>
+  <si>
+    <t>OS-079;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-10-09;2026-11-08;;Aberta;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-080;BCI-001;Bomba de incêndio;Predial;Preventiva;2026-10-09;2026-10-24;;Em andamento;Rafael Costa;Média</t>
+  </si>
+  <si>
+    <t>OS-081;CDR-001;Caldeira a vapor;Utilidades;Preventiva;2026-10-10;2026-10-25;;Aberta;Marcos Pereira;Baixa</t>
+  </si>
+  <si>
+    <t>OS-082;ELV-001;Elevador de carga;Predial;Preventiva;2026-10-10;2026-10-30;;Aberta;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-083;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-10-10;2026-10-17;;Aberta;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-084;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-10-11;2026-11-10;;Aberta;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-085;QDF-001;Quadro de distribuição A;Elétrica;Preventiva;2026-10-12;2026-10-19;;Em andamento;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-086;ELV-001;Elevador de carga;Predial;Preventiva;2026-10-13;2026-10-20;;Aberta;Rafael Costa;Alta</t>
+  </si>
+  <si>
+    <t>OS-087;GER-001;Gerador diesel;Elétrica;Preventiva;2026-10-15;2026-10-30;;Aberta;Marcos Pereira;Alta</t>
+  </si>
+  <si>
+    <t>OS-088;ELV-001;Elevador de carga;Predial;Preventiva;2026-10-15;2026-10-22;;Em andamento;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-089;PRS-001;Prensa hidráulica;Produção;Preventiva;2026-10-17;2026-10-27;;Aberta;Marcos Pereira;Média</t>
+  </si>
+  <si>
+    <t>OS-090;CMP-002;Compressor de ar 2;Utilidades;Preventiva;2026-10-17;2026-10-24;;Aberta;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-091;CMP-001;Compressor de ar 1;Utilidades;Preventiva;2026-10-18;2026-10-28;;Aberta;Paula Mendes;Baixa</t>
+  </si>
+  <si>
+    <t>OS-092;ARC-001;Ar-condicionado central;Predial;Preventiva;2026-10-21;2026-10-28;;Aberta;Juliana Alves;Média</t>
+  </si>
+  <si>
+    <t>OS-093;TRN-001;Torno CNC;Produção;Preventiva;2026-10-22;2026-11-11;;Aberta;Carlos Lima;Média</t>
+  </si>
+  <si>
+    <t>OS-094;BMB-003;Bomba dosadora;Utilidades;Preventiva;2026-10-24;2026-11-08;;Aberta;Carlos Lima;Alta</t>
+  </si>
+  <si>
+    <t>OS-095;BMB-001;Bomba centrífuga 1;Utilidades;Preventiva;2026-10-26;2026-11-05;;Aberta;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>OS-096;CMP-001;Compressor de ar 1;Utilidades;Preventiva;2026-10-26;2026-11-05;;Aberta;Rafael Costa;Média</t>
+  </si>
+  <si>
+    <t>OS-097;GER-001;Gerador diesel;Elétrica;Preventiva;2026-10-27;2026-11-03;;Aberta;Paula Mendes;Média</t>
+  </si>
+  <si>
+    <t>OS-098;ARC-002;Ar-condicionado split sala 2;Predial;Preventiva;2026-10-28;2026-11-07;;Aberta;Juliana Alves;Baixa</t>
+  </si>
+  <si>
+    <t>OS-099;EXA-001;Exaustor industrial;Produção;Preventiva;2026-10-29;2026-11-08;;Aberta;Ana Souza;Alta</t>
+  </si>
+  <si>
+    <t>OS-100;TRF-001;Transformador 500 kVA;Elétrica;Preventiva;2026-11-01;2026-11-08;;Aberta;Ana Souza;Média</t>
+  </si>
+  <si>
+    <t>STATUS DAS OS GERAL / RESPONSÁVEL</t>
   </si>
 </sst>
 </file>
@@ -1299,14 +1600,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="18" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1461,14 +1762,74 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>331096</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>373817</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Retângulo 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0CD6724-CF5F-074F-E0DD-6A9335DE5FD0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1495425" y="331096"/>
+          <a:ext cx="6591300" cy="42721"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="pt-BR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>161925</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>514350</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -1528,13 +1889,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>476252</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>2</xdr:row>
       <xdr:rowOff>66676</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>190499</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
@@ -1550,7 +1911,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1085852" y="1590676"/>
+          <a:off x="1085852" y="828676"/>
           <a:ext cx="1676398" cy="314323"/>
           <a:chOff x="1085852" y="1590676"/>
           <a:chExt cx="1676398" cy="314323"/>
@@ -1677,21 +2038,21 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>542925</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="16" name="Agrupar 15">
+        <xdr:cNvPr id="4" name="Agrupar 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA572593-528A-FACC-42D0-920B2E3F199B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82DB45B3-CD72-4A45-5A71-310EE81826CD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1699,149 +2060,18 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1428750" y="342900"/>
-          <a:ext cx="8058150" cy="581025"/>
-          <a:chOff x="1428750" y="342900"/>
+          <a:off x="1428750" y="0"/>
+          <a:ext cx="8058150" cy="542925"/>
+          <a:chOff x="1581150" y="323850"/>
           <a:chExt cx="8058150" cy="581025"/>
         </a:xfrm>
       </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="4" name="Agrupar 3">
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="3" name="CaixaDeTexto 2">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{82DB45B3-CD72-4A45-5A71-310EE81826CD}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="1428750" y="342900"/>
-            <a:ext cx="8058150" cy="581025"/>
-            <a:chOff x="1581150" y="323850"/>
-            <a:chExt cx="8058150" cy="581025"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="CaixaDeTexto 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF76171B-CD8D-2540-4AD5-0FF7744C6E05}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="1581150" y="323850"/>
-              <a:ext cx="8058150" cy="371475"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln w="9525" cmpd="sng">
-              <a:noFill/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="dk1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="pt-BR" sz="2400" b="1">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:rPr>
-                <a:t>Gestão de Manutenção Preventiva por Responsável</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="3" name="CaixaDeTexto 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79FC1DC9-5B16-7D10-0F30-48DEB00BC641}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="1600200" y="647700"/>
-              <a:ext cx="5400675" cy="257175"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln w="9525" cmpd="sng">
-              <a:noFill/>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="dk1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="pt-BR" i="1">
-                  <a:solidFill>
-                    <a:schemeClr val="bg1"/>
-                  </a:solidFill>
-                </a:rPr>
-                <a:t>Acompanhamento de ordens de serviço, prazos e status por responsável</a:t>
-              </a:r>
-              <a:endParaRPr lang="pt-BR" sz="1100" i="1">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:endParaRPr>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </xdr:grpSp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="6" name="CaixaDeTexto 5">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33AE54EB-A965-AFCE-FB67-B902993745E9}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79FC1DC9-5B16-7D10-0F30-48DEB00BC641}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1849,8 +2079,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="6372225" y="666750"/>
-            <a:ext cx="1057275" cy="219075"/>
+            <a:off x="1600200" y="647700"/>
+            <a:ext cx="5400675" cy="257175"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -1879,22 +2109,14 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
-              <a:rPr lang="pt-BR" sz="1100" b="0" i="1">
+              <a:rPr lang="pt-BR" i="1">
                 <a:solidFill>
                   <a:schemeClr val="bg1"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Atualizado</a:t>
+              <a:t>Acompanhamento de ordens de serviço, prazos e status por responsável</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="pt-BR" sz="1100" b="0" i="1" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t> em: </a:t>
-            </a:r>
-            <a:endParaRPr lang="pt-BR" sz="1100" b="0" i="1">
+            <a:endParaRPr lang="pt-BR" sz="1100" i="1">
               <a:solidFill>
                 <a:schemeClr val="bg1"/>
               </a:solidFill>
@@ -1902,12 +2124,12 @@
           </a:p>
         </xdr:txBody>
       </xdr:sp>
-      <xdr:sp macro="" textlink="AP3">
+      <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="11" name="CaixaDeTexto 10">
+          <xdr:cNvPr id="2" name="CaixaDeTexto 1">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2621725-7C04-4AE0-A2DA-67BA3B466B00}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF76171B-CD8D-2540-4AD5-0FF7744C6E05}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -1915,8 +2137,8 @@
         </xdr:nvSpPr>
         <xdr:spPr>
           <a:xfrm>
-            <a:off x="7286625" y="666750"/>
-            <a:ext cx="866775" cy="200025"/>
+            <a:off x="1581150" y="323850"/>
+            <a:ext cx="8058150" cy="371475"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -1944,72 +2166,163 @@
           <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
           <a:lstStyle/>
           <a:p>
-            <a:fld id="{82226BD8-8C80-4BAE-81B6-B26FDA9181C8}" type="TxLink">
-              <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:r>
+              <a:rPr lang="pt-BR" sz="2400" b="1">
                 <a:solidFill>
                   <a:schemeClr val="bg1"/>
                 </a:solidFill>
-                <a:latin typeface="Calibri"/>
-                <a:ea typeface="Calibri"/>
-                <a:cs typeface="Calibri"/>
               </a:rPr>
-              <a:pPr/>
-              <a:t>09/10/2026</a:t>
-            </a:fld>
-            <a:endParaRPr lang="pt-BR" sz="1100" b="0" i="1">
-              <a:solidFill>
-                <a:schemeClr val="bg1"/>
-              </a:solidFill>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="13" name="Retângulo 12">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0CD6724-CF5F-074F-E0DD-6A9335DE5FD0}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1495425" y="697231"/>
-            <a:ext cx="6591300" cy="45719"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="2">
-            <a:schemeClr val="accent1">
-              <a:shade val="15000"/>
-            </a:schemeClr>
-          </a:lnRef>
-          <a:fillRef idx="1">
-            <a:schemeClr val="accent1"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:schemeClr val="accent1"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="l"/>
-            <a:endParaRPr lang="pt-BR" sz="1100"/>
+              <a:t>Gestão de Manutenção Preventiva por Responsável</a:t>
+            </a:r>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
     </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>247651</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>302614</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1657351</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>552450</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="CaixaDeTexto 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33AE54EB-A965-AFCE-FB67-B902993745E9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6153151" y="302614"/>
+          <a:ext cx="1409700" cy="249836"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1100" b="0" i="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Data de referência:</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1381125</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>302614</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>489523</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="AP1">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="CaixaDeTexto 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F2621725-7C04-4AE0-A2DA-67BA3B466B00}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7286625" y="302614"/>
+          <a:ext cx="866775" cy="186909"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:fld id="{82226BD8-8C80-4BAE-81B6-B26FDA9181C8}" type="TxLink">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+              <a:ea typeface="Calibri"/>
+              <a:cs typeface="Calibri"/>
+            </a:rPr>
+            <a:pPr/>
+            <a:t>09/10/2026</a:t>
+          </a:fld>
+          <a:endParaRPr lang="pt-BR" sz="1100" b="0" i="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -2331,6 +2644,521 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D808016F-5910-4C3B-831D-609D3684589D}">
+  <dimension ref="A1:A101"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>269</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F7C0FA6-4804-4F52-95BC-5EEDAE952162}">
   <dimension ref="A1:K101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5759,9 +6587,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14B8D296-2926-4BF5-8E29-9FB41C0EEE9F}">
-  <dimension ref="C3:AP111"/>
+  <dimension ref="C1:AP107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="18.85546875" customWidth="1"/>
@@ -5774,2016 +6602,2013 @@
     <col min="42" max="42" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:42" s="17" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H3" s="26"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="AP3" s="27">
+    <row r="1" spans="3:42" s="17" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H1" s="26"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="AP1" s="27">
         <f ca="1">TODAY()</f>
         <v>46304</v>
       </c>
     </row>
-    <row r="8" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="19" t="s">
+    <row r="4" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C11" s="28" t="s">
-        <v>166</v>
-      </c>
-      <c r="D11" s="29"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="19" t="s">
+      <c r="D5" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E5" s="5"/>
+    </row>
+    <row r="6" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="29" t="s">
+        <v>270</v>
+      </c>
+      <c r="D7" s="30"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G7" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="H11" s="24" t="s">
+      <c r="H7" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="I11" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="J11" s="25" t="s">
+      <c r="I7" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="J7" s="25" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="20" t="s">
+    <row r="8" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="D12" s="21">
-        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C12),COUNTIFS(ordens_de_servico!J:J,resumo!D9,ordens_de_servico!I:I,resumo!C12))</f>
+      <c r="D8" s="21">
+        <f>IF($D$5="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C8),COUNTIFS(ordens_de_servico!J:J,resumo!$D$5,ordens_de_servico!I:I,resumo!C8))</f>
         <v>45</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12" s="7" t="s">
+      <c r="E8" s="1"/>
+      <c r="F8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H8" s="9">
         <v>46255</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I8" s="10">
         <f>IF(ordens_de_servico!H2&gt;ordens_de_servico!G2,-DATEDIF(ordens_de_servico!G2,ordens_de_servico!H2,"d"),IF(ordens_de_servico!H2=0,"",DATEDIF(ordens_de_servico!H2,ordens_de_servico!G2,"d")))</f>
         <v>-6</v>
       </c>
-      <c r="J12" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J2,ordens_de_servico!I2,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="20" t="s">
+      <c r="J8" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J2,ordens_de_servico!I2,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="21">
-        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C13),COUNTIFS(ordens_de_servico!J:J,resumo!D10,ordens_de_servico!I:I,resumo!C13))</f>
+      <c r="D9" s="21">
+        <f>IF($D$5="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C9),COUNTIFS(ordens_de_servico!J:J,resumo!$D$5,ordens_de_servico!I:I,resumo!C9))</f>
         <v>21</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13" s="7" t="s">
+      <c r="E9" s="1"/>
+      <c r="F9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H13" s="9">
+      <c r="H9" s="9">
         <v>46255</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I9" s="10">
         <f>IF(ordens_de_servico!H3&gt;ordens_de_servico!G3,-DATEDIF(ordens_de_servico!G3,ordens_de_servico!H3,"d"),IF(ordens_de_servico!H3=0,"",DATEDIF(ordens_de_servico!H3,ordens_de_servico!G3,"d")))</f>
         <v>2</v>
       </c>
-      <c r="J13" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J3,ordens_de_servico!I3,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="20" t="s">
+      <c r="J9" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J3,ordens_de_servico!I3,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="21">
-        <f>IF($D$9="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C14),COUNTIFS(ordens_de_servico!J:J,resumo!D11,ordens_de_servico!I:I,resumo!C14))</f>
+      <c r="D10" s="21">
+        <f>IF($D$5="Geral",COUNTIF(ordens_de_servico!I:I,resumo!C10),COUNTIFS(ordens_de_servico!J:J,resumo!$D$5,ordens_de_servico!I:I,resumo!C10))</f>
         <v>34</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="F14" s="7" t="s">
+      <c r="E10" s="1"/>
+      <c r="F10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="8" t="s">
+      <c r="G10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H10" s="9">
         <v>46257</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I10" s="10">
         <f>IF(ordens_de_servico!H4&gt;ordens_de_servico!G4,-DATEDIF(ordens_de_servico!G4,ordens_de_servico!H4,"d"),IF(ordens_de_servico!H4=0,"",DATEDIF(ordens_de_servico!H4,ordens_de_servico!G4,"d")))</f>
         <v>5</v>
       </c>
-      <c r="J14" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J4,ordens_de_servico!I4,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="D15" s="23">
-        <f>SUM(D12:D14)</f>
+      <c r="J10" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J4,ordens_de_servico!I4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="23">
+        <f>SUM(D8:D10)</f>
         <v>100</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="7" t="s">
+      <c r="E11" s="6"/>
+      <c r="F11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G15" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="9">
+      <c r="H11" s="9">
         <v>46248</v>
       </c>
-      <c r="I15" s="10">
+      <c r="I11" s="10">
         <f>IF(ordens_de_servico!H5&gt;ordens_de_servico!G5,-DATEDIF(ordens_de_servico!G5,ordens_de_servico!H5,"d"),IF(ordens_de_servico!H5=0,"",DATEDIF(ordens_de_servico!H5,ordens_de_servico!G5,"d")))</f>
         <v>3</v>
       </c>
-      <c r="J15" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J5,ordens_de_servico!I5,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="3"/>
-      <c r="F16" s="7" t="s">
+      <c r="J11" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J5,ordens_de_servico!I5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="3"/>
+      <c r="F12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="G16" s="8" t="s">
+      <c r="G12" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H16" s="9">
+      <c r="H12" s="9">
         <v>46246</v>
       </c>
-      <c r="I16" s="10">
+      <c r="I12" s="10">
         <f>IF(ordens_de_servico!H6&gt;ordens_de_servico!G6,-DATEDIF(ordens_de_servico!G6,ordens_de_servico!H6,"d"),IF(ordens_de_servico!H6=0,"",DATEDIF(ordens_de_servico!H6,ordens_de_servico!G6,"d")))</f>
         <v>5</v>
       </c>
+      <c r="J12" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J6,ordens_de_servico!I6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="1"/>
+      <c r="F13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H13" s="9">
+        <v>46254</v>
+      </c>
+      <c r="I13" s="10">
+        <f>IF(ordens_de_servico!H7&gt;ordens_de_servico!G7,-DATEDIF(ordens_de_servico!G7,ordens_de_servico!H7,"d"),IF(ordens_de_servico!H7=0,"",DATEDIF(ordens_de_servico!H7,ordens_de_servico!G7,"d")))</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J7,ordens_de_servico!I7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="1"/>
+      <c r="F14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="H14" s="9">
+        <v>46259</v>
+      </c>
+      <c r="I14" s="10">
+        <f>IF(ordens_de_servico!H8&gt;ordens_de_servico!G8,-DATEDIF(ordens_de_servico!G8,ordens_de_servico!H8,"d"),IF(ordens_de_servico!H8=0,"",DATEDIF(ordens_de_servico!H8,ordens_de_servico!G8,"d")))</f>
+        <v>5</v>
+      </c>
+      <c r="J14" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J8,ordens_de_servico!I8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="28"/>
+      <c r="F15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15" s="9">
+        <v>46247</v>
+      </c>
+      <c r="I15" s="10">
+        <f>IF(ordens_de_servico!H9&gt;ordens_de_servico!G9,-DATEDIF(ordens_de_servico!G9,ordens_de_servico!H9,"d"),IF(ordens_de_servico!H9=0,"",DATEDIF(ordens_de_servico!H9,ordens_de_servico!G9,"d")))</f>
+        <v>2</v>
+      </c>
+      <c r="J15" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J9,ordens_de_servico!I9,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="3:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="1"/>
+      <c r="F16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H16" s="9">
+        <v>46251</v>
+      </c>
+      <c r="I16" s="10">
+        <f>IF(ordens_de_servico!H10&gt;ordens_de_servico!G10,-DATEDIF(ordens_de_servico!G10,ordens_de_servico!H10,"d"),IF(ordens_de_servico!H10=0,"",DATEDIF(ordens_de_servico!H10,ordens_de_servico!G10,"d")))</f>
+        <v>1</v>
+      </c>
       <c r="J16" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J6,ordens_de_servico!I6,"")</f>
+        <f>IF($D$5=ordens_de_servico!J10,ordens_de_servico!I10,"")</f>
         <v/>
       </c>
     </row>
     <row r="17" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="1"/>
       <c r="F17" s="7" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H17" s="9">
-        <v>46254</v>
+        <v>46249</v>
       </c>
       <c r="I17" s="10">
-        <f>IF(ordens_de_servico!H7&gt;ordens_de_servico!G7,-DATEDIF(ordens_de_servico!G7,ordens_de_servico!H7,"d"),IF(ordens_de_servico!H7=0,"",DATEDIF(ordens_de_servico!H7,ordens_de_servico!G7,"d")))</f>
-        <v>0</v>
+        <f>IF(ordens_de_servico!H11&gt;ordens_de_servico!G11,-DATEDIF(ordens_de_servico!G11,ordens_de_servico!H11,"d"),IF(ordens_de_servico!H11=0,"",DATEDIF(ordens_de_servico!H11,ordens_de_servico!G11,"d")))</f>
+        <v>3</v>
       </c>
       <c r="J17" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J7,ordens_de_servico!I7,"")</f>
+        <f>IF($D$5=ordens_de_servico!J11,ordens_de_servico!I11,"")</f>
         <v/>
       </c>
     </row>
     <row r="18" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C18" s="1"/>
-      <c r="D18" t="s">
-        <v>169</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="H18" s="9">
-        <v>46259</v>
+        <v>46249</v>
       </c>
       <c r="I18" s="10">
-        <f>IF(ordens_de_servico!H8&gt;ordens_de_servico!G8,-DATEDIF(ordens_de_servico!G8,ordens_de_servico!H8,"d"),IF(ordens_de_servico!H8=0,"",DATEDIF(ordens_de_servico!H8,ordens_de_servico!G8,"d")))</f>
-        <v>5</v>
+        <f>IF(ordens_de_servico!H12&gt;ordens_de_servico!G12,-DATEDIF(ordens_de_servico!G12,ordens_de_servico!H12,"d"),IF(ordens_de_servico!H12=0,"",DATEDIF(ordens_de_servico!H12,ordens_de_servico!G12,"d")))</f>
+        <v>-6</v>
       </c>
       <c r="J18" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J8,ordens_de_servico!I8,"")</f>
+        <f>IF($D$5=ordens_de_servico!J12,ordens_de_servico!I12,"")</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="30"/>
       <c r="F19" s="7" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H19" s="9">
-        <v>46247</v>
+        <v>46254</v>
       </c>
       <c r="I19" s="10">
-        <f>IF(ordens_de_servico!H9&gt;ordens_de_servico!G9,-DATEDIF(ordens_de_servico!G9,ordens_de_servico!H9,"d"),IF(ordens_de_servico!H9=0,"",DATEDIF(ordens_de_servico!H9,ordens_de_servico!G9,"d")))</f>
+        <f>IF(ordens_de_servico!H13&gt;ordens_de_servico!G13,-DATEDIF(ordens_de_servico!G13,ordens_de_servico!H13,"d"),IF(ordens_de_servico!H13=0,"",DATEDIF(ordens_de_servico!H13,ordens_de_servico!G13,"d")))</f>
         <v>2</v>
       </c>
       <c r="J19" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J9,ordens_de_servico!I9,"")</f>
+        <f>IF($D$5=ordens_de_servico!J13,ordens_de_servico!I13,"")</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="1"/>
       <c r="F20" s="7" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="H20" s="9">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="I20" s="10">
-        <f>IF(ordens_de_servico!H10&gt;ordens_de_servico!G10,-DATEDIF(ordens_de_servico!G10,ordens_de_servico!H10,"d"),IF(ordens_de_servico!H10=0,"",DATEDIF(ordens_de_servico!H10,ordens_de_servico!G10,"d")))</f>
-        <v>1</v>
+        <f>IF(ordens_de_servico!H14&gt;ordens_de_servico!G14,-DATEDIF(ordens_de_servico!G14,ordens_de_servico!H14,"d"),IF(ordens_de_servico!H14=0,"",DATEDIF(ordens_de_servico!H14,ordens_de_servico!G14,"d")))</f>
+        <v>4</v>
       </c>
       <c r="J20" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J10,ordens_de_servico!I10,"")</f>
+        <f>IF($D$5=ordens_de_servico!J14,ordens_de_servico!I14,"")</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="1"/>
       <c r="F21" s="7" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>25</v>
       </c>
       <c r="H21" s="9">
-        <v>46249</v>
+        <v>46266</v>
       </c>
       <c r="I21" s="10">
-        <f>IF(ordens_de_servico!H11&gt;ordens_de_servico!G11,-DATEDIF(ordens_de_servico!G11,ordens_de_servico!H11,"d"),IF(ordens_de_servico!H11=0,"",DATEDIF(ordens_de_servico!H11,ordens_de_servico!G11,"d")))</f>
+        <f>IF(ordens_de_servico!H15&gt;ordens_de_servico!G15,-DATEDIF(ordens_de_servico!G15,ordens_de_servico!H15,"d"),IF(ordens_de_servico!H15=0,"",DATEDIF(ordens_de_servico!H15,ordens_de_servico!G15,"d")))</f>
+        <v>4</v>
+      </c>
+      <c r="J21" s="11" t="str">
+        <f>IF($D$5=ordens_de_servico!J15,ordens_de_servico!I15,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F22" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="H22" s="9">
+        <v>46256</v>
+      </c>
+      <c r="I22" s="10">
+        <f>IF(ordens_de_servico!H16&gt;ordens_de_servico!G16,-DATEDIF(ordens_de_servico!G16,ordens_de_servico!H16,"d"),IF(ordens_de_servico!H16=0,"",DATEDIF(ordens_de_servico!H16,ordens_de_servico!G16,"d")))</f>
         <v>3</v>
       </c>
-      <c r="J21" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J11,ordens_de_servico!I11,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="1"/>
-      <c r="F22" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H22" s="9">
-        <v>46249</v>
-      </c>
-      <c r="I22" s="10">
-        <f>IF(ordens_de_servico!H12&gt;ordens_de_servico!G12,-DATEDIF(ordens_de_servico!G12,ordens_de_servico!H12,"d"),IF(ordens_de_servico!H12=0,"",DATEDIF(ordens_de_servico!H12,ordens_de_servico!G12,"d")))</f>
-        <v>-6</v>
-      </c>
       <c r="J22" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J12,ordens_de_servico!I12,"")</f>
+        <f>IF($D$5=ordens_de_servico!J16,ordens_de_servico!I16,"")</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F23" s="7" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="H23" s="9">
-        <v>46254</v>
+        <v>46280</v>
       </c>
       <c r="I23" s="10">
-        <f>IF(ordens_de_servico!H13&gt;ordens_de_servico!G13,-DATEDIF(ordens_de_servico!G13,ordens_de_servico!H13,"d"),IF(ordens_de_servico!H13=0,"",DATEDIF(ordens_de_servico!H13,ordens_de_servico!G13,"d")))</f>
-        <v>2</v>
+        <f>IF(ordens_de_servico!H17&gt;ordens_de_servico!G17,-DATEDIF(ordens_de_servico!G17,ordens_de_servico!H17,"d"),IF(ordens_de_servico!H17=0,"",DATEDIF(ordens_de_servico!H17,ordens_de_servico!G17,"d")))</f>
+        <v>0</v>
       </c>
       <c r="J23" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J13,ordens_de_servico!I13,"")</f>
+        <f>IF($D$5=ordens_de_servico!J17,ordens_de_servico!I17,"")</f>
         <v/>
       </c>
     </row>
     <row r="24" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F24" s="7" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="H24" s="9">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="I24" s="10">
-        <f>IF(ordens_de_servico!H14&gt;ordens_de_servico!G14,-DATEDIF(ordens_de_servico!G14,ordens_de_servico!H14,"d"),IF(ordens_de_servico!H14=0,"",DATEDIF(ordens_de_servico!H14,ordens_de_servico!G14,"d")))</f>
-        <v>4</v>
+        <f>IF(ordens_de_servico!H18&gt;ordens_de_servico!G18,-DATEDIF(ordens_de_servico!G18,ordens_de_servico!H18,"d"),IF(ordens_de_servico!H18=0,"",DATEDIF(ordens_de_servico!H18,ordens_de_servico!G18,"d")))</f>
+        <v>3</v>
       </c>
       <c r="J24" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J14,ordens_de_servico!I14,"")</f>
+        <f>IF($D$5=ordens_de_servico!J18,ordens_de_servico!I18,"")</f>
         <v/>
       </c>
     </row>
     <row r="25" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F25" s="7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="H25" s="9">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="I25" s="10">
-        <f>IF(ordens_de_servico!H15&gt;ordens_de_servico!G15,-DATEDIF(ordens_de_servico!G15,ordens_de_servico!H15,"d"),IF(ordens_de_servico!H15=0,"",DATEDIF(ordens_de_servico!H15,ordens_de_servico!G15,"d")))</f>
-        <v>4</v>
+        <f>IF(ordens_de_servico!H19&gt;ordens_de_servico!G19,-DATEDIF(ordens_de_servico!G19,ordens_de_servico!H19,"d"),IF(ordens_de_servico!H19=0,"",DATEDIF(ordens_de_servico!H19,ordens_de_servico!G19,"d")))</f>
+        <v>0</v>
       </c>
       <c r="J25" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J15,ordens_de_servico!I15,"")</f>
+        <f>IF($D$5=ordens_de_servico!J19,ordens_de_servico!I19,"")</f>
         <v/>
       </c>
     </row>
     <row r="26" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F26" s="7" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="H26" s="9">
-        <v>46256</v>
+        <v>46273</v>
       </c>
       <c r="I26" s="10">
-        <f>IF(ordens_de_servico!H16&gt;ordens_de_servico!G16,-DATEDIF(ordens_de_servico!G16,ordens_de_servico!H16,"d"),IF(ordens_de_servico!H16=0,"",DATEDIF(ordens_de_servico!H16,ordens_de_servico!G16,"d")))</f>
-        <v>3</v>
+        <f>IF(ordens_de_servico!H20&gt;ordens_de_servico!G20,-DATEDIF(ordens_de_servico!G20,ordens_de_servico!H20,"d"),IF(ordens_de_servico!H20=0,"",DATEDIF(ordens_de_servico!H20,ordens_de_servico!G20,"d")))</f>
+        <v>-8</v>
       </c>
       <c r="J26" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J16,ordens_de_servico!I16,"")</f>
+        <f>IF($D$5=ordens_de_servico!J20,ordens_de_servico!I20,"")</f>
         <v/>
       </c>
     </row>
     <row r="27" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F27" s="7" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H27" s="9">
-        <v>46280</v>
+        <v>46260</v>
       </c>
       <c r="I27" s="10">
-        <f>IF(ordens_de_servico!H17&gt;ordens_de_servico!G17,-DATEDIF(ordens_de_servico!G17,ordens_de_servico!H17,"d"),IF(ordens_de_servico!H17=0,"",DATEDIF(ordens_de_servico!H17,ordens_de_servico!G17,"d")))</f>
-        <v>0</v>
+        <f>IF(ordens_de_servico!H21&gt;ordens_de_servico!G21,-DATEDIF(ordens_de_servico!G21,ordens_de_servico!H21,"d"),IF(ordens_de_servico!H21=0,"",DATEDIF(ordens_de_servico!H21,ordens_de_servico!G21,"d")))</f>
+        <v>3</v>
       </c>
       <c r="J27" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J17,ordens_de_servico!I17,"")</f>
+        <f>IF($D$5=ordens_de_servico!J21,ordens_de_servico!I21,"")</f>
         <v/>
       </c>
     </row>
     <row r="28" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F28" s="7" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="H28" s="9">
-        <v>46266</v>
+        <v>46261</v>
       </c>
       <c r="I28" s="10">
-        <f>IF(ordens_de_servico!H18&gt;ordens_de_servico!G18,-DATEDIF(ordens_de_servico!G18,ordens_de_servico!H18,"d"),IF(ordens_de_servico!H18=0,"",DATEDIF(ordens_de_servico!H18,ordens_de_servico!G18,"d")))</f>
-        <v>3</v>
+        <f>IF(ordens_de_servico!H22&gt;ordens_de_servico!G22,-DATEDIF(ordens_de_servico!G22,ordens_de_servico!H22,"d"),IF(ordens_de_servico!H22=0,"",DATEDIF(ordens_de_servico!H22,ordens_de_servico!G22,"d")))</f>
+        <v>-9</v>
       </c>
       <c r="J28" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J18,ordens_de_servico!I18,"")</f>
+        <f>IF($D$5=ordens_de_servico!J22,ordens_de_servico!I22,"")</f>
         <v/>
       </c>
     </row>
     <row r="29" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F29" s="7" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="H29" s="9">
-        <v>46262</v>
-      </c>
-      <c r="I29" s="10">
-        <f>IF(ordens_de_servico!H19&gt;ordens_de_servico!G19,-DATEDIF(ordens_de_servico!G19,ordens_de_servico!H19,"d"),IF(ordens_de_servico!H19=0,"",DATEDIF(ordens_de_servico!H19,ordens_de_servico!G19,"d")))</f>
-        <v>0</v>
+        <v>46274</v>
+      </c>
+      <c r="I29" s="10" t="str">
+        <f>IF(ordens_de_servico!H23&gt;ordens_de_servico!G23,-DATEDIF(ordens_de_servico!G23,ordens_de_servico!H23,"d"),IF(ordens_de_servico!H23=0,"",DATEDIF(ordens_de_servico!H23,ordens_de_servico!G23,"d")))</f>
+        <v/>
       </c>
       <c r="J29" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J19,ordens_de_servico!I19,"")</f>
+        <f>IF($D$5=ordens_de_servico!J23,ordens_de_servico!I23,"")</f>
         <v/>
       </c>
     </row>
     <row r="30" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F30" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G30" s="8" t="s">
         <v>72</v>
       </c>
       <c r="H30" s="9">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="I30" s="10">
-        <f>IF(ordens_de_servico!H20&gt;ordens_de_servico!G20,-DATEDIF(ordens_de_servico!G20,ordens_de_servico!H20,"d"),IF(ordens_de_servico!H20=0,"",DATEDIF(ordens_de_servico!H20,ordens_de_servico!G20,"d")))</f>
-        <v>-8</v>
+        <f>IF(ordens_de_servico!H24&gt;ordens_de_servico!G24,-DATEDIF(ordens_de_servico!G24,ordens_de_servico!H24,"d"),IF(ordens_de_servico!H24=0,"",DATEDIF(ordens_de_servico!H24,ordens_de_servico!G24,"d")))</f>
+        <v>1</v>
       </c>
       <c r="J30" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J20,ordens_de_servico!I20,"")</f>
+        <f>IF($D$5=ordens_de_servico!J24,ordens_de_servico!I24,"")</f>
         <v/>
       </c>
     </row>
     <row r="31" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F31" s="7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="H31" s="9">
-        <v>46260</v>
+        <v>46276</v>
       </c>
       <c r="I31" s="10">
-        <f>IF(ordens_de_servico!H21&gt;ordens_de_servico!G21,-DATEDIF(ordens_de_servico!G21,ordens_de_servico!H21,"d"),IF(ordens_de_servico!H21=0,"",DATEDIF(ordens_de_servico!H21,ordens_de_servico!G21,"d")))</f>
-        <v>3</v>
+        <f>IF(ordens_de_servico!H25&gt;ordens_de_servico!G25,-DATEDIF(ordens_de_servico!G25,ordens_de_servico!H25,"d"),IF(ordens_de_servico!H25=0,"",DATEDIF(ordens_de_servico!H25,ordens_de_servico!G25,"d")))</f>
+        <v>11</v>
       </c>
       <c r="J31" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J21,ordens_de_servico!I21,"")</f>
+        <f>IF($D$5=ordens_de_servico!J25,ordens_de_servico!I25,"")</f>
         <v/>
       </c>
     </row>
     <row r="32" spans="3:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F32" s="7" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="H32" s="9">
-        <v>46261</v>
+        <v>46267</v>
       </c>
       <c r="I32" s="10">
-        <f>IF(ordens_de_servico!H22&gt;ordens_de_servico!G22,-DATEDIF(ordens_de_servico!G22,ordens_de_servico!H22,"d"),IF(ordens_de_servico!H22=0,"",DATEDIF(ordens_de_servico!H22,ordens_de_servico!G22,"d")))</f>
-        <v>-9</v>
+        <f>IF(ordens_de_servico!H26&gt;ordens_de_servico!G26,-DATEDIF(ordens_de_servico!G26,ordens_de_servico!H26,"d"),IF(ordens_de_servico!H26=0,"",DATEDIF(ordens_de_servico!H26,ordens_de_servico!G26,"d")))</f>
+        <v>4</v>
       </c>
       <c r="J32" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J22,ordens_de_servico!I22,"")</f>
+        <f>IF($D$5=ordens_de_servico!J26,ordens_de_servico!I26,"")</f>
         <v/>
       </c>
     </row>
     <row r="33" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F33" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G33" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H33" s="9">
+        <v>46278</v>
+      </c>
+      <c r="I33" s="10">
+        <f>IF(ordens_de_servico!H27&gt;ordens_de_servico!G27,-DATEDIF(ordens_de_servico!G27,ordens_de_servico!H27,"d"),IF(ordens_de_servico!H27=0,"",DATEDIF(ordens_de_servico!H27,ordens_de_servico!G27,"d")))</f>
         <v>19</v>
       </c>
-      <c r="H33" s="9">
-        <v>46274</v>
-      </c>
-      <c r="I33" s="10" t="str">
-        <f>IF(ordens_de_servico!H23&gt;ordens_de_servico!G23,-DATEDIF(ordens_de_servico!G23,ordens_de_servico!H23,"d"),IF(ordens_de_servico!H23=0,"",DATEDIF(ordens_de_servico!H23,ordens_de_servico!G23,"d")))</f>
-        <v/>
-      </c>
       <c r="J33" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J23,ordens_de_servico!I23,"")</f>
+        <f>IF($D$5=ordens_de_servico!J27,ordens_de_servico!I27,"")</f>
         <v/>
       </c>
     </row>
     <row r="34" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F34" s="7" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>72</v>
+        <v>34</v>
       </c>
       <c r="H34" s="9">
-        <v>46276</v>
+        <v>46288</v>
       </c>
       <c r="I34" s="10">
-        <f>IF(ordens_de_servico!H24&gt;ordens_de_servico!G24,-DATEDIF(ordens_de_servico!G24,ordens_de_servico!H24,"d"),IF(ordens_de_servico!H24=0,"",DATEDIF(ordens_de_servico!H24,ordens_de_servico!G24,"d")))</f>
-        <v>1</v>
+        <f>IF(ordens_de_servico!H28&gt;ordens_de_servico!G28,-DATEDIF(ordens_de_servico!G28,ordens_de_servico!H28,"d"),IF(ordens_de_servico!H28=0,"",DATEDIF(ordens_de_servico!H28,ordens_de_servico!G28,"d")))</f>
+        <v>0</v>
       </c>
       <c r="J34" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J24,ordens_de_servico!I24,"")</f>
+        <f>IF($D$5=ordens_de_servico!J28,ordens_de_servico!I28,"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F35" s="7" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H35" s="9">
-        <v>46276</v>
-      </c>
-      <c r="I35" s="10">
-        <f>IF(ordens_de_servico!H25&gt;ordens_de_servico!G25,-DATEDIF(ordens_de_servico!G25,ordens_de_servico!H25,"d"),IF(ordens_de_servico!H25=0,"",DATEDIF(ordens_de_servico!H25,ordens_de_servico!G25,"d")))</f>
-        <v>11</v>
+        <v>46282</v>
+      </c>
+      <c r="I35" s="10" t="str">
+        <f>IF(ordens_de_servico!H29&gt;ordens_de_servico!G29,-DATEDIF(ordens_de_servico!G29,ordens_de_servico!H29,"d"),IF(ordens_de_servico!H29=0,"",DATEDIF(ordens_de_servico!H29,ordens_de_servico!G29,"d")))</f>
+        <v/>
       </c>
       <c r="J35" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J25,ordens_de_servico!I25,"")</f>
+        <f>IF($D$5=ordens_de_servico!J29,ordens_de_servico!I29,"")</f>
         <v/>
       </c>
     </row>
     <row r="36" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F36" s="7" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="H36" s="9">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="I36" s="10">
-        <f>IF(ordens_de_servico!H26&gt;ordens_de_servico!G26,-DATEDIF(ordens_de_servico!G26,ordens_de_servico!H26,"d"),IF(ordens_de_servico!H26=0,"",DATEDIF(ordens_de_servico!H26,ordens_de_servico!G26,"d")))</f>
-        <v>4</v>
+        <f>IF(ordens_de_servico!H30&gt;ordens_de_servico!G30,-DATEDIF(ordens_de_servico!G30,ordens_de_servico!H30,"d"),IF(ordens_de_servico!H30=0,"",DATEDIF(ordens_de_servico!H30,ordens_de_servico!G30,"d")))</f>
+        <v>6</v>
       </c>
       <c r="J36" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J26,ordens_de_servico!I26,"")</f>
+        <f>IF($D$5=ordens_de_servico!J30,ordens_de_servico!I30,"")</f>
         <v/>
       </c>
     </row>
     <row r="37" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F37" s="7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>65</v>
       </c>
       <c r="H37" s="9">
-        <v>46278</v>
-      </c>
-      <c r="I37" s="10">
-        <f>IF(ordens_de_servico!H27&gt;ordens_de_servico!G27,-DATEDIF(ordens_de_servico!G27,ordens_de_servico!H27,"d"),IF(ordens_de_servico!H27=0,"",DATEDIF(ordens_de_servico!H27,ordens_de_servico!G27,"d")))</f>
-        <v>19</v>
+        <v>46271</v>
+      </c>
+      <c r="I37" s="10" t="str">
+        <f>IF(ordens_de_servico!H31&gt;ordens_de_servico!G31,-DATEDIF(ordens_de_servico!G31,ordens_de_servico!H31,"d"),IF(ordens_de_servico!H31=0,"",DATEDIF(ordens_de_servico!H31,ordens_de_servico!G31,"d")))</f>
+        <v/>
       </c>
       <c r="J37" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J27,ordens_de_servico!I27,"")</f>
+        <f>IF($D$5=ordens_de_servico!J31,ordens_de_servico!I31,"")</f>
         <v/>
       </c>
     </row>
     <row r="38" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F38" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="H38" s="9">
-        <v>46288</v>
+        <v>46284</v>
       </c>
       <c r="I38" s="10">
-        <f>IF(ordens_de_servico!H28&gt;ordens_de_servico!G28,-DATEDIF(ordens_de_servico!G28,ordens_de_servico!H28,"d"),IF(ordens_de_servico!H28=0,"",DATEDIF(ordens_de_servico!H28,ordens_de_servico!G28,"d")))</f>
-        <v>0</v>
+        <f>IF(ordens_de_servico!H32&gt;ordens_de_servico!G32,-DATEDIF(ordens_de_servico!G32,ordens_de_servico!H32,"d"),IF(ordens_de_servico!H32=0,"",DATEDIF(ordens_de_servico!H32,ordens_de_servico!G32,"d")))</f>
+        <v>5</v>
       </c>
       <c r="J38" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J28,ordens_de_servico!I28,"")</f>
+        <f>IF($D$5=ordens_de_servico!J32,ordens_de_servico!I32,"")</f>
         <v/>
       </c>
     </row>
     <row r="39" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F39" s="7" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="H39" s="9">
-        <v>46282</v>
+        <v>46272</v>
       </c>
       <c r="I39" s="10" t="str">
-        <f>IF(ordens_de_servico!H29&gt;ordens_de_servico!G29,-DATEDIF(ordens_de_servico!G29,ordens_de_servico!H29,"d"),IF(ordens_de_servico!H29=0,"",DATEDIF(ordens_de_servico!H29,ordens_de_servico!G29,"d")))</f>
+        <f>IF(ordens_de_servico!H33&gt;ordens_de_servico!G33,-DATEDIF(ordens_de_servico!G33,ordens_de_servico!H33,"d"),IF(ordens_de_servico!H33=0,"",DATEDIF(ordens_de_servico!H33,ordens_de_servico!G33,"d")))</f>
         <v/>
       </c>
       <c r="J39" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J29,ordens_de_servico!I29,"")</f>
+        <f>IF($D$5=ordens_de_servico!J33,ordens_de_servico!I33,"")</f>
         <v/>
       </c>
     </row>
     <row r="40" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F40" s="7" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="H40" s="9">
-        <v>46269</v>
+        <v>46275</v>
       </c>
       <c r="I40" s="10">
-        <f>IF(ordens_de_servico!H30&gt;ordens_de_servico!G30,-DATEDIF(ordens_de_servico!G30,ordens_de_servico!H30,"d"),IF(ordens_de_servico!H30=0,"",DATEDIF(ordens_de_servico!H30,ordens_de_servico!G30,"d")))</f>
-        <v>6</v>
+        <f>IF(ordens_de_servico!H34&gt;ordens_de_servico!G34,-DATEDIF(ordens_de_servico!G34,ordens_de_servico!H34,"d"),IF(ordens_de_servico!H34=0,"",DATEDIF(ordens_de_servico!H34,ordens_de_servico!G34,"d")))</f>
+        <v>-2</v>
       </c>
       <c r="J40" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J30,ordens_de_servico!I30,"")</f>
+        <f>IF($D$5=ordens_de_servico!J34,ordens_de_servico!I34,"")</f>
         <v/>
       </c>
     </row>
     <row r="41" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F41" s="7" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G41" s="8" t="s">
         <v>65</v>
       </c>
       <c r="H41" s="9">
-        <v>46271</v>
+        <v>46276</v>
       </c>
       <c r="I41" s="10" t="str">
-        <f>IF(ordens_de_servico!H31&gt;ordens_de_servico!G31,-DATEDIF(ordens_de_servico!G31,ordens_de_servico!H31,"d"),IF(ordens_de_servico!H31=0,"",DATEDIF(ordens_de_servico!H31,ordens_de_servico!G31,"d")))</f>
+        <f>IF(ordens_de_servico!H35&gt;ordens_de_servico!G35,-DATEDIF(ordens_de_servico!G35,ordens_de_servico!H35,"d"),IF(ordens_de_servico!H35=0,"",DATEDIF(ordens_de_servico!H35,ordens_de_servico!G35,"d")))</f>
         <v/>
       </c>
       <c r="J41" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J31,ordens_de_servico!I31,"")</f>
+        <f>IF($D$5=ordens_de_servico!J35,ordens_de_servico!I35,"")</f>
         <v/>
       </c>
     </row>
     <row r="42" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F42" s="7" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="H42" s="9">
-        <v>46284</v>
-      </c>
-      <c r="I42" s="10">
-        <f>IF(ordens_de_servico!H32&gt;ordens_de_servico!G32,-DATEDIF(ordens_de_servico!G32,ordens_de_servico!H32,"d"),IF(ordens_de_servico!H32=0,"",DATEDIF(ordens_de_servico!H32,ordens_de_servico!G32,"d")))</f>
-        <v>5</v>
+        <v>46276</v>
+      </c>
+      <c r="I42" s="10" t="str">
+        <f>IF(ordens_de_servico!H36&gt;ordens_de_servico!G36,-DATEDIF(ordens_de_servico!G36,ordens_de_servico!H36,"d"),IF(ordens_de_servico!H36=0,"",DATEDIF(ordens_de_servico!H36,ordens_de_servico!G36,"d")))</f>
+        <v/>
       </c>
       <c r="J42" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J32,ordens_de_servico!I32,"")</f>
+        <f>IF($D$5=ordens_de_servico!J36,ordens_de_servico!I36,"")</f>
         <v/>
       </c>
     </row>
     <row r="43" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F43" s="7" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="H43" s="9">
-        <v>46272</v>
-      </c>
-      <c r="I43" s="10" t="str">
-        <f>IF(ordens_de_servico!H33&gt;ordens_de_servico!G33,-DATEDIF(ordens_de_servico!G33,ordens_de_servico!H33,"d"),IF(ordens_de_servico!H33=0,"",DATEDIF(ordens_de_servico!H33,ordens_de_servico!G33,"d")))</f>
-        <v/>
+        <v>46282</v>
+      </c>
+      <c r="I43" s="10">
+        <f>IF(ordens_de_servico!H37&gt;ordens_de_servico!G37,-DATEDIF(ordens_de_servico!G37,ordens_de_servico!H37,"d"),IF(ordens_de_servico!H37=0,"",DATEDIF(ordens_de_servico!H37,ordens_de_servico!G37,"d")))</f>
+        <v>5</v>
       </c>
       <c r="J43" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J33,ordens_de_servico!I33,"")</f>
+        <f>IF($D$5=ordens_de_servico!J37,ordens_de_servico!I37,"")</f>
         <v/>
       </c>
     </row>
     <row r="44" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F44" s="7" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="H44" s="9">
-        <v>46275</v>
-      </c>
-      <c r="I44" s="10">
-        <f>IF(ordens_de_servico!H34&gt;ordens_de_servico!G34,-DATEDIF(ordens_de_servico!G34,ordens_de_servico!H34,"d"),IF(ordens_de_servico!H34=0,"",DATEDIF(ordens_de_servico!H34,ordens_de_servico!G34,"d")))</f>
-        <v>-2</v>
+        <v>46287</v>
+      </c>
+      <c r="I44" s="10" t="str">
+        <f>IF(ordens_de_servico!H38&gt;ordens_de_servico!G38,-DATEDIF(ordens_de_servico!G38,ordens_de_servico!H38,"d"),IF(ordens_de_servico!H38=0,"",DATEDIF(ordens_de_servico!H38,ordens_de_servico!G38,"d")))</f>
+        <v/>
       </c>
       <c r="J44" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J34,ordens_de_servico!I34,"")</f>
+        <f>IF($D$5=ordens_de_servico!J38,ordens_de_servico!I38,"")</f>
         <v/>
       </c>
     </row>
     <row r="45" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F45" s="7" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>65</v>
+        <v>19</v>
       </c>
       <c r="H45" s="9">
-        <v>46276</v>
-      </c>
-      <c r="I45" s="10" t="str">
-        <f>IF(ordens_de_servico!H35&gt;ordens_de_servico!G35,-DATEDIF(ordens_de_servico!G35,ordens_de_servico!H35,"d"),IF(ordens_de_servico!H35=0,"",DATEDIF(ordens_de_servico!H35,ordens_de_servico!G35,"d")))</f>
-        <v/>
+        <v>46288</v>
+      </c>
+      <c r="I45" s="10">
+        <f>IF(ordens_de_servico!H39&gt;ordens_de_servico!G39,-DATEDIF(ordens_de_servico!G39,ordens_de_servico!H39,"d"),IF(ordens_de_servico!H39=0,"",DATEDIF(ordens_de_servico!H39,ordens_de_servico!G39,"d")))</f>
+        <v>-83</v>
       </c>
       <c r="J45" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J35,ordens_de_servico!I35,"")</f>
+        <f>IF($D$5=ordens_de_servico!J39,ordens_de_servico!I39,"")</f>
         <v/>
       </c>
     </row>
     <row r="46" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F46" s="7" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="H46" s="9">
-        <v>46276</v>
-      </c>
-      <c r="I46" s="10" t="str">
-        <f>IF(ordens_de_servico!H36&gt;ordens_de_servico!G36,-DATEDIF(ordens_de_servico!G36,ordens_de_servico!H36,"d"),IF(ordens_de_servico!H36=0,"",DATEDIF(ordens_de_servico!H36,ordens_de_servico!G36,"d")))</f>
-        <v/>
+        <v>46283</v>
+      </c>
+      <c r="I46" s="10">
+        <f>IF(ordens_de_servico!H40&gt;ordens_de_servico!G40,-DATEDIF(ordens_de_servico!G40,ordens_de_servico!H40,"d"),IF(ordens_de_servico!H40=0,"",DATEDIF(ordens_de_servico!H40,ordens_de_servico!G40,"d")))</f>
+        <v>-47</v>
       </c>
       <c r="J46" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J36,ordens_de_servico!I36,"")</f>
+        <f>IF($D$5=ordens_de_servico!J40,ordens_de_servico!I40,"")</f>
         <v/>
       </c>
     </row>
     <row r="47" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F47" s="7" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="H47" s="9">
-        <v>46282</v>
-      </c>
-      <c r="I47" s="10">
-        <f>IF(ordens_de_servico!H37&gt;ordens_de_servico!G37,-DATEDIF(ordens_de_servico!G37,ordens_de_servico!H37,"d"),IF(ordens_de_servico!H37=0,"",DATEDIF(ordens_de_servico!H37,ordens_de_servico!G37,"d")))</f>
-        <v>5</v>
+        <v>46303</v>
+      </c>
+      <c r="I47" s="10" t="str">
+        <f>IF(ordens_de_servico!H41&gt;ordens_de_servico!G41,-DATEDIF(ordens_de_servico!G41,ordens_de_servico!H41,"d"),IF(ordens_de_servico!H41=0,"",DATEDIF(ordens_de_servico!H41,ordens_de_servico!G41,"d")))</f>
+        <v/>
       </c>
       <c r="J47" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J37,ordens_de_servico!I37,"")</f>
+        <f>IF($D$5=ordens_de_servico!J41,ordens_de_servico!I41,"")</f>
         <v/>
       </c>
     </row>
     <row r="48" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F48" s="7" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="H48" s="9">
-        <v>46287</v>
-      </c>
-      <c r="I48" s="10" t="str">
-        <f>IF(ordens_de_servico!H38&gt;ordens_de_servico!G38,-DATEDIF(ordens_de_servico!G38,ordens_de_servico!H38,"d"),IF(ordens_de_servico!H38=0,"",DATEDIF(ordens_de_servico!H38,ordens_de_servico!G38,"d")))</f>
-        <v/>
+        <v>46283</v>
+      </c>
+      <c r="I48" s="10">
+        <f>IF(ordens_de_servico!H42&gt;ordens_de_servico!G42,-DATEDIF(ordens_de_servico!G42,ordens_de_servico!H42,"d"),IF(ordens_de_servico!H42=0,"",DATEDIF(ordens_de_servico!H42,ordens_de_servico!G42,"d")))</f>
+        <v>1</v>
       </c>
       <c r="J48" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J38,ordens_de_servico!I38,"")</f>
+        <f>IF($D$5=ordens_de_servico!J42,ordens_de_servico!I42,"")</f>
         <v/>
       </c>
     </row>
     <row r="49" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F49" s="7" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="H49" s="9">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="I49" s="10">
-        <f>IF(ordens_de_servico!H39&gt;ordens_de_servico!G39,-DATEDIF(ordens_de_servico!G39,ordens_de_servico!H39,"d"),IF(ordens_de_servico!H39=0,"",DATEDIF(ordens_de_servico!H39,ordens_de_servico!G39,"d")))</f>
-        <v>-83</v>
+        <f>IF(ordens_de_servico!H43&gt;ordens_de_servico!G43,-DATEDIF(ordens_de_servico!G43,ordens_de_servico!H43,"d"),IF(ordens_de_servico!H43=0,"",DATEDIF(ordens_de_servico!H43,ordens_de_servico!G43,"d")))</f>
+        <v>-3</v>
       </c>
       <c r="J49" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J39,ordens_de_servico!I39,"")</f>
+        <f>IF($D$5=ordens_de_servico!J43,ordens_de_servico!I43,"")</f>
         <v/>
       </c>
     </row>
     <row r="50" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F50" s="7" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="H50" s="9">
-        <v>46283</v>
-      </c>
-      <c r="I50" s="10">
-        <f>IF(ordens_de_servico!H40&gt;ordens_de_servico!G40,-DATEDIF(ordens_de_servico!G40,ordens_de_servico!H40,"d"),IF(ordens_de_servico!H40=0,"",DATEDIF(ordens_de_servico!H40,ordens_de_servico!G40,"d")))</f>
-        <v>-47</v>
+        <v>46281</v>
+      </c>
+      <c r="I50" s="10" t="str">
+        <f>IF(ordens_de_servico!H44&gt;ordens_de_servico!G44,-DATEDIF(ordens_de_servico!G44,ordens_de_servico!H44,"d"),IF(ordens_de_servico!H44=0,"",DATEDIF(ordens_de_servico!H44,ordens_de_servico!G44,"d")))</f>
+        <v/>
       </c>
       <c r="J50" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J40,ordens_de_servico!I40,"")</f>
+        <f>IF($D$5=ordens_de_servico!J44,ordens_de_servico!I44,"")</f>
         <v/>
       </c>
     </row>
     <row r="51" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F51" s="7" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="G51" s="8" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H51" s="9">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="I51" s="10" t="str">
-        <f>IF(ordens_de_servico!H41&gt;ordens_de_servico!G41,-DATEDIF(ordens_de_servico!G41,ordens_de_servico!H41,"d"),IF(ordens_de_servico!H41=0,"",DATEDIF(ordens_de_servico!H41,ordens_de_servico!G41,"d")))</f>
+        <f>IF(ordens_de_servico!H45&gt;ordens_de_servico!G45,-DATEDIF(ordens_de_servico!G45,ordens_de_servico!H45,"d"),IF(ordens_de_servico!H45=0,"",DATEDIF(ordens_de_servico!H45,ordens_de_servico!G45,"d")))</f>
         <v/>
       </c>
       <c r="J51" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J41,ordens_de_servico!I41,"")</f>
+        <f>IF($D$5=ordens_de_servico!J45,ordens_de_servico!I45,"")</f>
         <v/>
       </c>
     </row>
     <row r="52" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F52" s="7" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="H52" s="9">
-        <v>46283</v>
-      </c>
-      <c r="I52" s="10">
-        <f>IF(ordens_de_servico!H42&gt;ordens_de_servico!G42,-DATEDIF(ordens_de_servico!G42,ordens_de_servico!H42,"d"),IF(ordens_de_servico!H42=0,"",DATEDIF(ordens_de_servico!H42,ordens_de_servico!G42,"d")))</f>
-        <v>1</v>
+        <v>46304</v>
+      </c>
+      <c r="I52" s="10" t="str">
+        <f>IF(ordens_de_servico!H46&gt;ordens_de_servico!G46,-DATEDIF(ordens_de_servico!G46,ordens_de_servico!H46,"d"),IF(ordens_de_servico!H46=0,"",DATEDIF(ordens_de_servico!H46,ordens_de_servico!G46,"d")))</f>
+        <v/>
       </c>
       <c r="J52" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J42,ordens_de_servico!I42,"")</f>
+        <f>IF($D$5=ordens_de_servico!J46,ordens_de_servico!I46,"")</f>
         <v/>
       </c>
     </row>
     <row r="53" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F53" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="H53" s="9">
-        <v>46283</v>
-      </c>
-      <c r="I53" s="10">
-        <f>IF(ordens_de_servico!H43&gt;ordens_de_servico!G43,-DATEDIF(ordens_de_servico!G43,ordens_de_servico!H43,"d"),IF(ordens_de_servico!H43=0,"",DATEDIF(ordens_de_servico!H43,ordens_de_servico!G43,"d")))</f>
-        <v>-3</v>
+        <v>46304</v>
+      </c>
+      <c r="I53" s="10" t="str">
+        <f>IF(ordens_de_servico!H47&gt;ordens_de_servico!G47,-DATEDIF(ordens_de_servico!G47,ordens_de_servico!H47,"d"),IF(ordens_de_servico!H47=0,"",DATEDIF(ordens_de_servico!H47,ordens_de_servico!G47,"d")))</f>
+        <v/>
       </c>
       <c r="J53" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J43,ordens_de_servico!I43,"")</f>
+        <f>IF($D$5=ordens_de_servico!J47,ordens_de_servico!I47,"")</f>
         <v/>
       </c>
     </row>
     <row r="54" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F54" s="7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="G54" s="8" t="s">
-        <v>37</v>
+        <v>108</v>
       </c>
       <c r="H54" s="9">
-        <v>46281</v>
+        <v>46304</v>
       </c>
       <c r="I54" s="10" t="str">
-        <f>IF(ordens_de_servico!H44&gt;ordens_de_servico!G44,-DATEDIF(ordens_de_servico!G44,ordens_de_servico!H44,"d"),IF(ordens_de_servico!H44=0,"",DATEDIF(ordens_de_servico!H44,ordens_de_servico!G44,"d")))</f>
+        <f>IF(ordens_de_servico!H48&gt;ordens_de_servico!G48,-DATEDIF(ordens_de_servico!G48,ordens_de_servico!H48,"d"),IF(ordens_de_servico!H48=0,"",DATEDIF(ordens_de_servico!H48,ordens_de_servico!G48,"d")))</f>
         <v/>
       </c>
       <c r="J54" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J44,ordens_de_servico!I44,"")</f>
+        <f>IF($D$5=ordens_de_servico!J48,ordens_de_servico!I48,"")</f>
         <v/>
       </c>
     </row>
     <row r="55" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F55" s="7" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="H55" s="9">
-        <v>46304</v>
+        <v>46297</v>
       </c>
       <c r="I55" s="10" t="str">
-        <f>IF(ordens_de_servico!H45&gt;ordens_de_servico!G45,-DATEDIF(ordens_de_servico!G45,ordens_de_servico!H45,"d"),IF(ordens_de_servico!H45=0,"",DATEDIF(ordens_de_servico!H45,ordens_de_servico!G45,"d")))</f>
+        <f>IF(ordens_de_servico!H49&gt;ordens_de_servico!G49,-DATEDIF(ordens_de_servico!G49,ordens_de_servico!H49,"d"),IF(ordens_de_servico!H49=0,"",DATEDIF(ordens_de_servico!H49,ordens_de_servico!G49,"d")))</f>
         <v/>
       </c>
       <c r="J55" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J45,ordens_de_servico!I45,"")</f>
+        <f>IF($D$5=ordens_de_servico!J49,ordens_de_servico!I49,"")</f>
         <v/>
       </c>
     </row>
     <row r="56" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F56" s="7" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="H56" s="9">
-        <v>46304</v>
+        <v>46294</v>
       </c>
       <c r="I56" s="10" t="str">
-        <f>IF(ordens_de_servico!H46&gt;ordens_de_servico!G46,-DATEDIF(ordens_de_servico!G46,ordens_de_servico!H46,"d"),IF(ordens_de_servico!H46=0,"",DATEDIF(ordens_de_servico!H46,ordens_de_servico!G46,"d")))</f>
+        <f>IF(ordens_de_servico!H50&gt;ordens_de_servico!G50,-DATEDIF(ordens_de_servico!G50,ordens_de_servico!H50,"d"),IF(ordens_de_servico!H50=0,"",DATEDIF(ordens_de_servico!H50,ordens_de_servico!G50,"d")))</f>
         <v/>
       </c>
       <c r="J56" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J46,ordens_de_servico!I46,"")</f>
+        <f>IF($D$5=ordens_de_servico!J50,ordens_de_servico!I50,"")</f>
         <v/>
       </c>
     </row>
     <row r="57" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F57" s="7" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="H57" s="9">
-        <v>46304</v>
+        <v>46310</v>
       </c>
       <c r="I57" s="10" t="str">
-        <f>IF(ordens_de_servico!H47&gt;ordens_de_servico!G47,-DATEDIF(ordens_de_servico!G47,ordens_de_servico!H47,"d"),IF(ordens_de_servico!H47=0,"",DATEDIF(ordens_de_servico!H47,ordens_de_servico!G47,"d")))</f>
+        <f>IF(ordens_de_servico!H51&gt;ordens_de_servico!G51,-DATEDIF(ordens_de_servico!G51,ordens_de_servico!H51,"d"),IF(ordens_de_servico!H51=0,"",DATEDIF(ordens_de_servico!H51,ordens_de_servico!G51,"d")))</f>
         <v/>
       </c>
       <c r="J57" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J47,ordens_de_servico!I47,"")</f>
+        <f>IF($D$5=ordens_de_servico!J51,ordens_de_servico!I51,"")</f>
         <v/>
       </c>
     </row>
     <row r="58" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F58" s="7" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="G58" s="8" t="s">
         <v>108</v>
       </c>
       <c r="H58" s="9">
-        <v>46304</v>
+        <v>46289</v>
       </c>
       <c r="I58" s="10" t="str">
-        <f>IF(ordens_de_servico!H48&gt;ordens_de_servico!G48,-DATEDIF(ordens_de_servico!G48,ordens_de_servico!H48,"d"),IF(ordens_de_servico!H48=0,"",DATEDIF(ordens_de_servico!H48,ordens_de_servico!G48,"d")))</f>
+        <f>IF(ordens_de_servico!H52&gt;ordens_de_servico!G52,-DATEDIF(ordens_de_servico!G52,ordens_de_servico!H52,"d"),IF(ordens_de_servico!H52=0,"",DATEDIF(ordens_de_servico!H52,ordens_de_servico!G52,"d")))</f>
         <v/>
       </c>
       <c r="J58" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J48,ordens_de_servico!I48,"")</f>
+        <f>IF($D$5=ordens_de_servico!J52,ordens_de_servico!I52,"")</f>
         <v/>
       </c>
     </row>
     <row r="59" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F59" s="7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="H59" s="9">
-        <v>46297</v>
+        <v>46303</v>
       </c>
       <c r="I59" s="10" t="str">
-        <f>IF(ordens_de_servico!H49&gt;ordens_de_servico!G49,-DATEDIF(ordens_de_servico!G49,ordens_de_servico!H49,"d"),IF(ordens_de_servico!H49=0,"",DATEDIF(ordens_de_servico!H49,ordens_de_servico!G49,"d")))</f>
+        <f>IF(ordens_de_servico!H53&gt;ordens_de_servico!G53,-DATEDIF(ordens_de_servico!G53,ordens_de_servico!H53,"d"),IF(ordens_de_servico!H53=0,"",DATEDIF(ordens_de_servico!H53,ordens_de_servico!G53,"d")))</f>
         <v/>
       </c>
       <c r="J59" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J49,ordens_de_servico!I49,"")</f>
+        <f>IF($D$5=ordens_de_servico!J53,ordens_de_servico!I53,"")</f>
         <v/>
       </c>
     </row>
     <row r="60" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F60" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G60" s="8" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="H60" s="9">
-        <v>46294</v>
+        <v>46301</v>
       </c>
       <c r="I60" s="10" t="str">
-        <f>IF(ordens_de_servico!H50&gt;ordens_de_servico!G50,-DATEDIF(ordens_de_servico!G50,ordens_de_servico!H50,"d"),IF(ordens_de_servico!H50=0,"",DATEDIF(ordens_de_servico!H50,ordens_de_servico!G50,"d")))</f>
+        <f>IF(ordens_de_servico!H54&gt;ordens_de_servico!G54,-DATEDIF(ordens_de_servico!G54,ordens_de_servico!H54,"d"),IF(ordens_de_servico!H54=0,"",DATEDIF(ordens_de_servico!H54,ordens_de_servico!G54,"d")))</f>
         <v/>
       </c>
       <c r="J60" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J50,ordens_de_servico!I50,"")</f>
+        <f>IF($D$5=ordens_de_servico!J54,ordens_de_servico!I54,"")</f>
         <v/>
       </c>
     </row>
     <row r="61" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F61" s="7" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="H61" s="9">
-        <v>46310</v>
+        <v>46302</v>
       </c>
       <c r="I61" s="10" t="str">
-        <f>IF(ordens_de_servico!H51&gt;ordens_de_servico!G51,-DATEDIF(ordens_de_servico!G51,ordens_de_servico!H51,"d"),IF(ordens_de_servico!H51=0,"",DATEDIF(ordens_de_servico!H51,ordens_de_servico!G51,"d")))</f>
+        <f>IF(ordens_de_servico!H55&gt;ordens_de_servico!G55,-DATEDIF(ordens_de_servico!G55,ordens_de_servico!H55,"d"),IF(ordens_de_servico!H55=0,"",DATEDIF(ordens_de_servico!H55,ordens_de_servico!G55,"d")))</f>
         <v/>
       </c>
       <c r="J61" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J51,ordens_de_servico!I51,"")</f>
+        <f>IF($D$5=ordens_de_servico!J55,ordens_de_servico!I55,"")</f>
         <v/>
       </c>
     </row>
     <row r="62" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F62" s="7" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>108</v>
+        <v>34</v>
       </c>
       <c r="H62" s="9">
-        <v>46289</v>
+        <v>46309</v>
       </c>
       <c r="I62" s="10" t="str">
-        <f>IF(ordens_de_servico!H52&gt;ordens_de_servico!G52,-DATEDIF(ordens_de_servico!G52,ordens_de_servico!H52,"d"),IF(ordens_de_servico!H52=0,"",DATEDIF(ordens_de_servico!H52,ordens_de_servico!G52,"d")))</f>
+        <f>IF(ordens_de_servico!H56&gt;ordens_de_servico!G56,-DATEDIF(ordens_de_servico!G56,ordens_de_servico!H56,"d"),IF(ordens_de_servico!H56=0,"",DATEDIF(ordens_de_servico!H56,ordens_de_servico!G56,"d")))</f>
         <v/>
       </c>
       <c r="J62" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J52,ordens_de_servico!I52,"")</f>
+        <f>IF($D$5=ordens_de_servico!J56,ordens_de_servico!I56,"")</f>
         <v/>
       </c>
     </row>
     <row r="63" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F63" s="7" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="H63" s="9">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="I63" s="10" t="str">
-        <f>IF(ordens_de_servico!H53&gt;ordens_de_servico!G53,-DATEDIF(ordens_de_servico!G53,ordens_de_servico!H53,"d"),IF(ordens_de_servico!H53=0,"",DATEDIF(ordens_de_servico!H53,ordens_de_servico!G53,"d")))</f>
+        <f>IF(ordens_de_servico!H57&gt;ordens_de_servico!G57,-DATEDIF(ordens_de_servico!G57,ordens_de_servico!H57,"d"),IF(ordens_de_servico!H57=0,"",DATEDIF(ordens_de_servico!H57,ordens_de_servico!G57,"d")))</f>
         <v/>
       </c>
       <c r="J63" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J53,ordens_de_servico!I53,"")</f>
+        <f>IF($D$5=ordens_de_servico!J57,ordens_de_servico!I57,"")</f>
         <v/>
       </c>
     </row>
     <row r="64" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F64" s="7" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="G64" s="8" t="s">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="H64" s="9">
-        <v>46301</v>
+        <v>46320</v>
       </c>
       <c r="I64" s="10" t="str">
-        <f>IF(ordens_de_servico!H54&gt;ordens_de_servico!G54,-DATEDIF(ordens_de_servico!G54,ordens_de_servico!H54,"d"),IF(ordens_de_servico!H54=0,"",DATEDIF(ordens_de_servico!H54,ordens_de_servico!G54,"d")))</f>
+        <f>IF(ordens_de_servico!H58&gt;ordens_de_servico!G58,-DATEDIF(ordens_de_servico!G58,ordens_de_servico!H58,"d"),IF(ordens_de_servico!H58=0,"",DATEDIF(ordens_de_servico!H58,ordens_de_servico!G58,"d")))</f>
         <v/>
       </c>
       <c r="J64" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J54,ordens_de_servico!I54,"")</f>
+        <f>IF($D$5=ordens_de_servico!J58,ordens_de_servico!I58,"")</f>
         <v/>
       </c>
     </row>
     <row r="65" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F65" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="H65" s="9">
-        <v>46302</v>
+        <v>46310</v>
       </c>
       <c r="I65" s="10" t="str">
-        <f>IF(ordens_de_servico!H55&gt;ordens_de_servico!G55,-DATEDIF(ordens_de_servico!G55,ordens_de_servico!H55,"d"),IF(ordens_de_servico!H55=0,"",DATEDIF(ordens_de_servico!H55,ordens_de_servico!G55,"d")))</f>
+        <f>IF(ordens_de_servico!H59&gt;ordens_de_servico!G59,-DATEDIF(ordens_de_servico!G59,ordens_de_servico!H59,"d"),IF(ordens_de_servico!H59=0,"",DATEDIF(ordens_de_servico!H59,ordens_de_servico!G59,"d")))</f>
         <v/>
       </c>
       <c r="J65" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J55,ordens_de_servico!I55,"")</f>
+        <f>IF($D$5=ordens_de_servico!J59,ordens_de_servico!I59,"")</f>
         <v/>
       </c>
     </row>
     <row r="66" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F66" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="G66" s="8" t="s">
         <v>34</v>
       </c>
       <c r="H66" s="9">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="I66" s="10" t="str">
-        <f>IF(ordens_de_servico!H56&gt;ordens_de_servico!G56,-DATEDIF(ordens_de_servico!G56,ordens_de_servico!H56,"d"),IF(ordens_de_servico!H56=0,"",DATEDIF(ordens_de_servico!H56,ordens_de_servico!G56,"d")))</f>
+        <f>IF(ordens_de_servico!H60&gt;ordens_de_servico!G60,-DATEDIF(ordens_de_servico!G60,ordens_de_servico!H60,"d"),IF(ordens_de_servico!H60=0,"",DATEDIF(ordens_de_servico!H60,ordens_de_servico!G60,"d")))</f>
         <v/>
       </c>
       <c r="J66" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J56,ordens_de_servico!I56,"")</f>
+        <f>IF($D$5=ordens_de_servico!J60,ordens_de_servico!I60,"")</f>
         <v/>
       </c>
     </row>
     <row r="67" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F67" s="7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>56</v>
+        <v>108</v>
       </c>
       <c r="H67" s="9">
-        <v>46300</v>
+        <v>46306</v>
       </c>
       <c r="I67" s="10" t="str">
-        <f>IF(ordens_de_servico!H57&gt;ordens_de_servico!G57,-DATEDIF(ordens_de_servico!G57,ordens_de_servico!H57,"d"),IF(ordens_de_servico!H57=0,"",DATEDIF(ordens_de_servico!H57,ordens_de_servico!G57,"d")))</f>
+        <f>IF(ordens_de_servico!H61&gt;ordens_de_servico!G61,-DATEDIF(ordens_de_servico!G61,ordens_de_servico!H61,"d"),IF(ordens_de_servico!H61=0,"",DATEDIF(ordens_de_servico!H61,ordens_de_servico!G61,"d")))</f>
         <v/>
       </c>
       <c r="J67" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J57,ordens_de_servico!I57,"")</f>
+        <f>IF($D$5=ordens_de_servico!J61,ordens_de_servico!I61,"")</f>
         <v/>
       </c>
     </row>
     <row r="68" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F68" s="7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="G68" s="8" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="H68" s="9">
-        <v>46320</v>
+        <v>46298</v>
       </c>
       <c r="I68" s="10" t="str">
-        <f>IF(ordens_de_servico!H58&gt;ordens_de_servico!G58,-DATEDIF(ordens_de_servico!G58,ordens_de_servico!H58,"d"),IF(ordens_de_servico!H58=0,"",DATEDIF(ordens_de_servico!H58,ordens_de_servico!G58,"d")))</f>
+        <f>IF(ordens_de_servico!H62&gt;ordens_de_servico!G62,-DATEDIF(ordens_de_servico!G62,ordens_de_servico!H62,"d"),IF(ordens_de_servico!H62=0,"",DATEDIF(ordens_de_servico!H62,ordens_de_servico!G62,"d")))</f>
         <v/>
       </c>
       <c r="J68" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J58,ordens_de_servico!I58,"")</f>
+        <f>IF($D$5=ordens_de_servico!J62,ordens_de_servico!I62,"")</f>
         <v/>
       </c>
     </row>
     <row r="69" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F69" s="7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="H69" s="9">
-        <v>46310</v>
+        <v>46301</v>
       </c>
       <c r="I69" s="10" t="str">
-        <f>IF(ordens_de_servico!H59&gt;ordens_de_servico!G59,-DATEDIF(ordens_de_servico!G59,ordens_de_servico!H59,"d"),IF(ordens_de_servico!H59=0,"",DATEDIF(ordens_de_servico!H59,ordens_de_servico!G59,"d")))</f>
+        <f>IF(ordens_de_servico!H63&gt;ordens_de_servico!G63,-DATEDIF(ordens_de_servico!G63,ordens_de_servico!H63,"d"),IF(ordens_de_servico!H63=0,"",DATEDIF(ordens_de_servico!H63,ordens_de_servico!G63,"d")))</f>
         <v/>
       </c>
       <c r="J69" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J59,ordens_de_servico!I59,"")</f>
+        <f>IF($D$5=ordens_de_servico!J63,ordens_de_servico!I63,"")</f>
         <v/>
       </c>
     </row>
     <row r="70" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F70" s="7" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G70" s="8" t="s">
-        <v>34</v>
+        <v>100</v>
       </c>
       <c r="H70" s="9">
         <v>46311</v>
       </c>
       <c r="I70" s="10" t="str">
-        <f>IF(ordens_de_servico!H60&gt;ordens_de_servico!G60,-DATEDIF(ordens_de_servico!G60,ordens_de_servico!H60,"d"),IF(ordens_de_servico!H60=0,"",DATEDIF(ordens_de_servico!H60,ordens_de_servico!G60,"d")))</f>
+        <f>IF(ordens_de_servico!H64&gt;ordens_de_servico!G64,-DATEDIF(ordens_de_servico!G64,ordens_de_servico!H64,"d"),IF(ordens_de_servico!H64=0,"",DATEDIF(ordens_de_servico!H64,ordens_de_servico!G64,"d")))</f>
         <v/>
       </c>
       <c r="J70" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J60,ordens_de_servico!I60,"")</f>
+        <f>IF($D$5=ordens_de_servico!J64,ordens_de_servico!I64,"")</f>
         <v/>
       </c>
     </row>
     <row r="71" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F71" s="7" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G71" s="8" t="s">
         <v>108</v>
       </c>
       <c r="H71" s="9">
-        <v>46306</v>
+        <v>46301</v>
       </c>
       <c r="I71" s="10" t="str">
-        <f>IF(ordens_de_servico!H61&gt;ordens_de_servico!G61,-DATEDIF(ordens_de_servico!G61,ordens_de_servico!H61,"d"),IF(ordens_de_servico!H61=0,"",DATEDIF(ordens_de_servico!H61,ordens_de_servico!G61,"d")))</f>
+        <f>IF(ordens_de_servico!H65&gt;ordens_de_servico!G65,-DATEDIF(ordens_de_servico!G65,ordens_de_servico!H65,"d"),IF(ordens_de_servico!H65=0,"",DATEDIF(ordens_de_servico!H65,ordens_de_servico!G65,"d")))</f>
         <v/>
       </c>
       <c r="J71" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J61,ordens_de_servico!I61,"")</f>
+        <f>IF($D$5=ordens_de_servico!J65,ordens_de_servico!I65,"")</f>
         <v/>
       </c>
     </row>
     <row r="72" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F72" s="7" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G72" s="8" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="H72" s="9">
-        <v>46298</v>
+        <v>46322</v>
       </c>
       <c r="I72" s="10" t="str">
-        <f>IF(ordens_de_servico!H62&gt;ordens_de_servico!G62,-DATEDIF(ordens_de_servico!G62,ordens_de_servico!H62,"d"),IF(ordens_de_servico!H62=0,"",DATEDIF(ordens_de_servico!H62,ordens_de_servico!G62,"d")))</f>
+        <f>IF(ordens_de_servico!H66&gt;ordens_de_servico!G66,-DATEDIF(ordens_de_servico!G66,ordens_de_servico!H66,"d"),IF(ordens_de_servico!H66=0,"",DATEDIF(ordens_de_servico!H66,ordens_de_servico!G66,"d")))</f>
         <v/>
       </c>
       <c r="J72" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J62,ordens_de_servico!I62,"")</f>
+        <f>IF($D$5=ordens_de_servico!J66,ordens_de_servico!I66,"")</f>
         <v/>
       </c>
     </row>
     <row r="73" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F73" s="7" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="H73" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="I73" s="10" t="str">
-        <f>IF(ordens_de_servico!H63&gt;ordens_de_servico!G63,-DATEDIF(ordens_de_servico!G63,ordens_de_servico!H63,"d"),IF(ordens_de_servico!H63=0,"",DATEDIF(ordens_de_servico!H63,ordens_de_servico!G63,"d")))</f>
+        <f>IF(ordens_de_servico!H67&gt;ordens_de_servico!G67,-DATEDIF(ordens_de_servico!G67,ordens_de_servico!H67,"d"),IF(ordens_de_servico!H67=0,"",DATEDIF(ordens_de_servico!H67,ordens_de_servico!G67,"d")))</f>
         <v/>
       </c>
       <c r="J73" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J63,ordens_de_servico!I63,"")</f>
+        <f>IF($D$5=ordens_de_servico!J67,ordens_de_servico!I67,"")</f>
         <v/>
       </c>
     </row>
     <row r="74" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F74" s="7" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G74" s="8" t="s">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="H74" s="9">
-        <v>46311</v>
+        <v>46303</v>
       </c>
       <c r="I74" s="10" t="str">
-        <f>IF(ordens_de_servico!H64&gt;ordens_de_servico!G64,-DATEDIF(ordens_de_servico!G64,ordens_de_servico!H64,"d"),IF(ordens_de_servico!H64=0,"",DATEDIF(ordens_de_servico!H64,ordens_de_servico!G64,"d")))</f>
+        <f>IF(ordens_de_servico!H68&gt;ordens_de_servico!G68,-DATEDIF(ordens_de_servico!G68,ordens_de_servico!H68,"d"),IF(ordens_de_servico!H68=0,"",DATEDIF(ordens_de_servico!H68,ordens_de_servico!G68,"d")))</f>
         <v/>
       </c>
       <c r="J74" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J64,ordens_de_servico!I64,"")</f>
+        <f>IF($D$5=ordens_de_servico!J68,ordens_de_servico!I68,"")</f>
         <v/>
       </c>
     </row>
     <row r="75" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F75" s="7" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>108</v>
+        <v>62</v>
       </c>
       <c r="H75" s="9">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="I75" s="10" t="str">
-        <f>IF(ordens_de_servico!H65&gt;ordens_de_servico!G65,-DATEDIF(ordens_de_servico!G65,ordens_de_servico!H65,"d"),IF(ordens_de_servico!H65=0,"",DATEDIF(ordens_de_servico!H65,ordens_de_servico!G65,"d")))</f>
+        <f>IF(ordens_de_servico!H69&gt;ordens_de_servico!G69,-DATEDIF(ordens_de_servico!G69,ordens_de_servico!H69,"d"),IF(ordens_de_servico!H69=0,"",DATEDIF(ordens_de_servico!H69,ordens_de_servico!G69,"d")))</f>
         <v/>
       </c>
       <c r="J75" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J65,ordens_de_servico!I65,"")</f>
+        <f>IF($D$5=ordens_de_servico!J69,ordens_de_servico!I69,"")</f>
         <v/>
       </c>
     </row>
     <row r="76" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F76" s="7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="G76" s="8" t="s">
-        <v>45</v>
+        <v>108</v>
       </c>
       <c r="H76" s="9">
-        <v>46322</v>
+        <v>46313</v>
       </c>
       <c r="I76" s="10" t="str">
-        <f>IF(ordens_de_servico!H66&gt;ordens_de_servico!G66,-DATEDIF(ordens_de_servico!G66,ordens_de_servico!H66,"d"),IF(ordens_de_servico!H66=0,"",DATEDIF(ordens_de_servico!H66,ordens_de_servico!G66,"d")))</f>
+        <f>IF(ordens_de_servico!H70&gt;ordens_de_servico!G70,-DATEDIF(ordens_de_servico!G70,ordens_de_servico!H70,"d"),IF(ordens_de_servico!H70=0,"",DATEDIF(ordens_de_servico!H70,ordens_de_servico!G70,"d")))</f>
         <v/>
       </c>
       <c r="J76" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J66,ordens_de_servico!I66,"")</f>
+        <f>IF($D$5=ordens_de_servico!J70,ordens_de_servico!I70,"")</f>
         <v/>
       </c>
     </row>
     <row r="77" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F77" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="H77" s="9">
-        <v>46300</v>
+        <v>46324</v>
       </c>
       <c r="I77" s="10" t="str">
-        <f>IF(ordens_de_servico!H67&gt;ordens_de_servico!G67,-DATEDIF(ordens_de_servico!G67,ordens_de_servico!H67,"d"),IF(ordens_de_servico!H67=0,"",DATEDIF(ordens_de_servico!H67,ordens_de_servico!G67,"d")))</f>
+        <f>IF(ordens_de_servico!H71&gt;ordens_de_servico!G71,-DATEDIF(ordens_de_servico!G71,ordens_de_servico!H71,"d"),IF(ordens_de_servico!H71=0,"",DATEDIF(ordens_de_servico!H71,ordens_de_servico!G71,"d")))</f>
         <v/>
       </c>
       <c r="J77" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J67,ordens_de_servico!I67,"")</f>
+        <f>IF($D$5=ordens_de_servico!J71,ordens_de_servico!I71,"")</f>
         <v/>
       </c>
     </row>
     <row r="78" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F78" s="7" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="G78" s="8" t="s">
-        <v>45</v>
+        <v>116</v>
       </c>
       <c r="H78" s="9">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="I78" s="10" t="str">
-        <f>IF(ordens_de_servico!H68&gt;ordens_de_servico!G68,-DATEDIF(ordens_de_servico!G68,ordens_de_servico!H68,"d"),IF(ordens_de_servico!H68=0,"",DATEDIF(ordens_de_servico!H68,ordens_de_servico!G68,"d")))</f>
+        <f>IF(ordens_de_servico!H72&gt;ordens_de_servico!G72,-DATEDIF(ordens_de_servico!G72,ordens_de_servico!H72,"d"),IF(ordens_de_servico!H72=0,"",DATEDIF(ordens_de_servico!H72,ordens_de_servico!G72,"d")))</f>
         <v/>
       </c>
       <c r="J78" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J68,ordens_de_servico!I68,"")</f>
+        <f>IF($D$5=ordens_de_servico!J72,ordens_de_servico!I72,"")</f>
         <v/>
       </c>
     </row>
     <row r="79" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F79" s="7" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="G79" s="8" t="s">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="H79" s="9">
-        <v>46300</v>
+        <v>46310</v>
       </c>
       <c r="I79" s="10" t="str">
-        <f>IF(ordens_de_servico!H69&gt;ordens_de_servico!G69,-DATEDIF(ordens_de_servico!G69,ordens_de_servico!H69,"d"),IF(ordens_de_servico!H69=0,"",DATEDIF(ordens_de_servico!H69,ordens_de_servico!G69,"d")))</f>
+        <f>IF(ordens_de_servico!H73&gt;ordens_de_servico!G73,-DATEDIF(ordens_de_servico!G73,ordens_de_servico!H73,"d"),IF(ordens_de_servico!H73=0,"",DATEDIF(ordens_de_servico!H73,ordens_de_servico!G73,"d")))</f>
         <v/>
       </c>
       <c r="J79" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J69,ordens_de_servico!I69,"")</f>
+        <f>IF($D$5=ordens_de_servico!J73,ordens_de_servico!I73,"")</f>
         <v/>
       </c>
     </row>
     <row r="80" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F80" s="7" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G80" s="8" t="s">
-        <v>108</v>
+        <v>45</v>
       </c>
       <c r="H80" s="9">
-        <v>46313</v>
+        <v>46305</v>
       </c>
       <c r="I80" s="10" t="str">
-        <f>IF(ordens_de_servico!H70&gt;ordens_de_servico!G70,-DATEDIF(ordens_de_servico!G70,ordens_de_servico!H70,"d"),IF(ordens_de_servico!H70=0,"",DATEDIF(ordens_de_servico!H70,ordens_de_servico!G70,"d")))</f>
+        <f>IF(ordens_de_servico!H74&gt;ordens_de_servico!G74,-DATEDIF(ordens_de_servico!G74,ordens_de_servico!H74,"d"),IF(ordens_de_servico!H74=0,"",DATEDIF(ordens_de_servico!H74,ordens_de_servico!G74,"d")))</f>
         <v/>
       </c>
       <c r="J80" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J70,ordens_de_servico!I70,"")</f>
+        <f>IF($D$5=ordens_de_servico!J74,ordens_de_servico!I74,"")</f>
         <v/>
       </c>
     </row>
     <row r="81" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F81" s="7" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="G81" s="8" t="s">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="H81" s="9">
-        <v>46324</v>
+        <v>46304</v>
       </c>
       <c r="I81" s="10" t="str">
-        <f>IF(ordens_de_servico!H71&gt;ordens_de_servico!G71,-DATEDIF(ordens_de_servico!G71,ordens_de_servico!H71,"d"),IF(ordens_de_servico!H71=0,"",DATEDIF(ordens_de_servico!H71,ordens_de_servico!G71,"d")))</f>
+        <f>IF(ordens_de_servico!H75&gt;ordens_de_servico!G75,-DATEDIF(ordens_de_servico!G75,ordens_de_servico!H75,"d"),IF(ordens_de_servico!H75=0,"",DATEDIF(ordens_de_servico!H75,ordens_de_servico!G75,"d")))</f>
         <v/>
       </c>
       <c r="J81" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J71,ordens_de_servico!I71,"")</f>
+        <f>IF($D$5=ordens_de_servico!J75,ordens_de_servico!I75,"")</f>
         <v/>
       </c>
     </row>
     <row r="82" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F82" s="7" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G82" s="8" t="s">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="H82" s="9">
-        <v>46304</v>
+        <v>46328</v>
       </c>
       <c r="I82" s="10" t="str">
-        <f>IF(ordens_de_servico!H72&gt;ordens_de_servico!G72,-DATEDIF(ordens_de_servico!G72,ordens_de_servico!H72,"d"),IF(ordens_de_servico!H72=0,"",DATEDIF(ordens_de_servico!H72,ordens_de_servico!G72,"d")))</f>
+        <f>IF(ordens_de_servico!H76&gt;ordens_de_servico!G76,-DATEDIF(ordens_de_servico!G76,ordens_de_servico!H76,"d"),IF(ordens_de_servico!H76=0,"",DATEDIF(ordens_de_servico!H76,ordens_de_servico!G76,"d")))</f>
         <v/>
       </c>
       <c r="J82" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J72,ordens_de_servico!I72,"")</f>
+        <f>IF($D$5=ordens_de_servico!J76,ordens_de_servico!I76,"")</f>
         <v/>
       </c>
     </row>
     <row r="83" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F83" s="7" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="H83" s="9">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="I83" s="10" t="str">
-        <f>IF(ordens_de_servico!H73&gt;ordens_de_servico!G73,-DATEDIF(ordens_de_servico!G73,ordens_de_servico!H73,"d"),IF(ordens_de_servico!H73=0,"",DATEDIF(ordens_de_servico!H73,ordens_de_servico!G73,"d")))</f>
+        <f>IF(ordens_de_servico!H77&gt;ordens_de_servico!G77,-DATEDIF(ordens_de_servico!G77,ordens_de_servico!H77,"d"),IF(ordens_de_servico!H77=0,"",DATEDIF(ordens_de_servico!H77,ordens_de_servico!G77,"d")))</f>
         <v/>
       </c>
       <c r="J83" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J73,ordens_de_servico!I73,"")</f>
+        <f>IF($D$5=ordens_de_servico!J77,ordens_de_servico!I77,"")</f>
         <v/>
       </c>
     </row>
     <row r="84" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F84" s="7" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="G84" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="H84" s="9">
-        <v>46305</v>
+        <v>46310</v>
       </c>
       <c r="I84" s="10" t="str">
-        <f>IF(ordens_de_servico!H74&gt;ordens_de_servico!G74,-DATEDIF(ordens_de_servico!G74,ordens_de_servico!H74,"d"),IF(ordens_de_servico!H74=0,"",DATEDIF(ordens_de_servico!H74,ordens_de_servico!G74,"d")))</f>
+        <f>IF(ordens_de_servico!H78&gt;ordens_de_servico!G78,-DATEDIF(ordens_de_servico!G78,ordens_de_servico!H78,"d"),IF(ordens_de_servico!H78=0,"",DATEDIF(ordens_de_servico!H78,ordens_de_servico!G78,"d")))</f>
         <v/>
       </c>
       <c r="J84" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J74,ordens_de_servico!I74,"")</f>
+        <f>IF($D$5=ordens_de_servico!J78,ordens_de_servico!I78,"")</f>
         <v/>
       </c>
     </row>
     <row r="85" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F85" s="7" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="G85" s="8" t="s">
         <v>34</v>
       </c>
       <c r="H85" s="9">
-        <v>46304</v>
+        <v>46322</v>
       </c>
       <c r="I85" s="10" t="str">
-        <f>IF(ordens_de_servico!H75&gt;ordens_de_servico!G75,-DATEDIF(ordens_de_servico!G75,ordens_de_servico!H75,"d"),IF(ordens_de_servico!H75=0,"",DATEDIF(ordens_de_servico!H75,ordens_de_servico!G75,"d")))</f>
+        <f>IF(ordens_de_servico!H79&gt;ordens_de_servico!G79,-DATEDIF(ordens_de_servico!G79,ordens_de_servico!H79,"d"),IF(ordens_de_servico!H79=0,"",DATEDIF(ordens_de_servico!H79,ordens_de_servico!G79,"d")))</f>
         <v/>
       </c>
       <c r="J85" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J75,ordens_de_servico!I75,"")</f>
+        <f>IF($D$5=ordens_de_servico!J79,ordens_de_servico!I79,"")</f>
         <v/>
       </c>
     </row>
     <row r="86" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F86" s="7" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="H86" s="9">
-        <v>46328</v>
+        <v>46334</v>
       </c>
       <c r="I86" s="10" t="str">
-        <f>IF(ordens_de_servico!H76&gt;ordens_de_servico!G76,-DATEDIF(ordens_de_servico!G76,ordens_de_servico!H76,"d"),IF(ordens_de_servico!H76=0,"",DATEDIF(ordens_de_servico!H76,ordens_de_servico!G76,"d")))</f>
+        <f>IF(ordens_de_servico!H80&gt;ordens_de_servico!G80,-DATEDIF(ordens_de_servico!G80,ordens_de_servico!H80,"d"),IF(ordens_de_servico!H80=0,"",DATEDIF(ordens_de_servico!H80,ordens_de_servico!G80,"d")))</f>
         <v/>
       </c>
       <c r="J86" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J76,ordens_de_servico!I76,"")</f>
+        <f>IF($D$5=ordens_de_servico!J80,ordens_de_servico!I80,"")</f>
         <v/>
       </c>
     </row>
     <row r="87" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F87" s="7" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="H87" s="9">
-        <v>46309</v>
+        <v>46319</v>
       </c>
       <c r="I87" s="10" t="str">
-        <f>IF(ordens_de_servico!H77&gt;ordens_de_servico!G77,-DATEDIF(ordens_de_servico!G77,ordens_de_servico!H77,"d"),IF(ordens_de_servico!H77=0,"",DATEDIF(ordens_de_servico!H77,ordens_de_servico!G77,"d")))</f>
+        <f>IF(ordens_de_servico!H81&gt;ordens_de_servico!G81,-DATEDIF(ordens_de_servico!G81,ordens_de_servico!H81,"d"),IF(ordens_de_servico!H81=0,"",DATEDIF(ordens_de_servico!H81,ordens_de_servico!G81,"d")))</f>
         <v/>
       </c>
       <c r="J87" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J77,ordens_de_servico!I77,"")</f>
+        <f>IF($D$5=ordens_de_servico!J81,ordens_de_servico!I81,"")</f>
         <v/>
       </c>
     </row>
     <row r="88" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F88" s="7" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G88" s="8" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="H88" s="9">
-        <v>46310</v>
+        <v>46320</v>
       </c>
       <c r="I88" s="10" t="str">
-        <f>IF(ordens_de_servico!H78&gt;ordens_de_servico!G78,-DATEDIF(ordens_de_servico!G78,ordens_de_servico!H78,"d"),IF(ordens_de_servico!H78=0,"",DATEDIF(ordens_de_servico!H78,ordens_de_servico!G78,"d")))</f>
+        <f>IF(ordens_de_servico!H82&gt;ordens_de_servico!G82,-DATEDIF(ordens_de_servico!G82,ordens_de_servico!H82,"d"),IF(ordens_de_servico!H82=0,"",DATEDIF(ordens_de_servico!H82,ordens_de_servico!G82,"d")))</f>
         <v/>
       </c>
       <c r="J88" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J78,ordens_de_servico!I78,"")</f>
+        <f>IF($D$5=ordens_de_servico!J82,ordens_de_servico!I82,"")</f>
         <v/>
       </c>
     </row>
     <row r="89" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F89" s="7" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="G89" s="8" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="H89" s="9">
-        <v>46322</v>
+        <v>46325</v>
       </c>
       <c r="I89" s="10" t="str">
-        <f>IF(ordens_de_servico!H79&gt;ordens_de_servico!G79,-DATEDIF(ordens_de_servico!G79,ordens_de_servico!H79,"d"),IF(ordens_de_servico!H79=0,"",DATEDIF(ordens_de_servico!H79,ordens_de_servico!G79,"d")))</f>
+        <f>IF(ordens_de_servico!H83&gt;ordens_de_servico!G83,-DATEDIF(ordens_de_servico!G83,ordens_de_servico!H83,"d"),IF(ordens_de_servico!H83=0,"",DATEDIF(ordens_de_servico!H83,ordens_de_servico!G83,"d")))</f>
         <v/>
       </c>
       <c r="J89" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J79,ordens_de_servico!I79,"")</f>
+        <f>IF($D$5=ordens_de_servico!J83,ordens_de_servico!I83,"")</f>
         <v/>
       </c>
     </row>
     <row r="90" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F90" s="7" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G90" s="8" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="H90" s="9">
-        <v>46334</v>
+        <v>46312</v>
       </c>
       <c r="I90" s="10" t="str">
-        <f>IF(ordens_de_servico!H80&gt;ordens_de_servico!G80,-DATEDIF(ordens_de_servico!G80,ordens_de_servico!H80,"d"),IF(ordens_de_servico!H80=0,"",DATEDIF(ordens_de_servico!H80,ordens_de_servico!G80,"d")))</f>
+        <f>IF(ordens_de_servico!H84&gt;ordens_de_servico!G84,-DATEDIF(ordens_de_servico!G84,ordens_de_servico!H84,"d"),IF(ordens_de_servico!H84=0,"",DATEDIF(ordens_de_servico!H84,ordens_de_servico!G84,"d")))</f>
         <v/>
       </c>
       <c r="J90" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J80,ordens_de_servico!I80,"")</f>
+        <f>IF($D$5=ordens_de_servico!J84,ordens_de_servico!I84,"")</f>
         <v/>
       </c>
     </row>
     <row r="91" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F91" s="7" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H91" s="9">
-        <v>46319</v>
+        <v>46336</v>
       </c>
       <c r="I91" s="10" t="str">
-        <f>IF(ordens_de_servico!H81&gt;ordens_de_servico!G81,-DATEDIF(ordens_de_servico!G81,ordens_de_servico!H81,"d"),IF(ordens_de_servico!H81=0,"",DATEDIF(ordens_de_servico!H81,ordens_de_servico!G81,"d")))</f>
+        <f>IF(ordens_de_servico!H85&gt;ordens_de_servico!G85,-DATEDIF(ordens_de_servico!G85,ordens_de_servico!H85,"d"),IF(ordens_de_servico!H85=0,"",DATEDIF(ordens_de_servico!H85,ordens_de_servico!G85,"d")))</f>
         <v/>
       </c>
       <c r="J91" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J81,ordens_de_servico!I81,"")</f>
+        <f>IF($D$5=ordens_de_servico!J85,ordens_de_servico!I85,"")</f>
         <v/>
       </c>
     </row>
     <row r="92" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F92" s="7" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="G92" s="8" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H92" s="9">
-        <v>46320</v>
+        <v>46314</v>
       </c>
       <c r="I92" s="10" t="str">
-        <f>IF(ordens_de_servico!H82&gt;ordens_de_servico!G82,-DATEDIF(ordens_de_servico!G82,ordens_de_servico!H82,"d"),IF(ordens_de_servico!H82=0,"",DATEDIF(ordens_de_servico!H82,ordens_de_servico!G82,"d")))</f>
+        <f>IF(ordens_de_servico!H86&gt;ordens_de_servico!G86,-DATEDIF(ordens_de_servico!G86,ordens_de_servico!H86,"d"),IF(ordens_de_servico!H86=0,"",DATEDIF(ordens_de_servico!H86,ordens_de_servico!G86,"d")))</f>
         <v/>
       </c>
       <c r="J92" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J82,ordens_de_servico!I82,"")</f>
+        <f>IF($D$5=ordens_de_servico!J86,ordens_de_servico!I86,"")</f>
         <v/>
       </c>
     </row>
     <row r="93" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F93" s="7" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="G93" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H93" s="9">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="I93" s="10" t="str">
-        <f>IF(ordens_de_servico!H83&gt;ordens_de_servico!G83,-DATEDIF(ordens_de_servico!G83,ordens_de_servico!H83,"d"),IF(ordens_de_servico!H83=0,"",DATEDIF(ordens_de_servico!H83,ordens_de_servico!G83,"d")))</f>
+        <f>IF(ordens_de_servico!H87&gt;ordens_de_servico!G87,-DATEDIF(ordens_de_servico!G87,ordens_de_servico!H87,"d"),IF(ordens_de_servico!H87=0,"",DATEDIF(ordens_de_servico!H87,ordens_de_servico!G87,"d")))</f>
         <v/>
       </c>
       <c r="J93" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J83,ordens_de_servico!I83,"")</f>
+        <f>IF($D$5=ordens_de_servico!J87,ordens_de_servico!I87,"")</f>
         <v/>
       </c>
     </row>
     <row r="94" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F94" s="7" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H94" s="9">
-        <v>46312</v>
+        <v>46325</v>
       </c>
       <c r="I94" s="10" t="str">
-        <f>IF(ordens_de_servico!H84&gt;ordens_de_servico!G84,-DATEDIF(ordens_de_servico!G84,ordens_de_servico!H84,"d"),IF(ordens_de_servico!H84=0,"",DATEDIF(ordens_de_servico!H84,ordens_de_servico!G84,"d")))</f>
+        <f>IF(ordens_de_servico!H88&gt;ordens_de_servico!G88,-DATEDIF(ordens_de_servico!G88,ordens_de_servico!H88,"d"),IF(ordens_de_servico!H88=0,"",DATEDIF(ordens_de_servico!H88,ordens_de_servico!G88,"d")))</f>
         <v/>
       </c>
       <c r="J94" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J84,ordens_de_servico!I84,"")</f>
+        <f>IF($D$5=ordens_de_servico!J88,ordens_de_servico!I88,"")</f>
         <v/>
       </c>
     </row>
     <row r="95" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F95" s="7" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="G95" s="8" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="H95" s="9">
-        <v>46336</v>
+        <v>46317</v>
       </c>
       <c r="I95" s="10" t="str">
-        <f>IF(ordens_de_servico!H85&gt;ordens_de_servico!G85,-DATEDIF(ordens_de_servico!G85,ordens_de_servico!H85,"d"),IF(ordens_de_servico!H85=0,"",DATEDIF(ordens_de_servico!H85,ordens_de_servico!G85,"d")))</f>
+        <f>IF(ordens_de_servico!H89&gt;ordens_de_servico!G89,-DATEDIF(ordens_de_servico!G89,ordens_de_servico!H89,"d"),IF(ordens_de_servico!H89=0,"",DATEDIF(ordens_de_servico!H89,ordens_de_servico!G89,"d")))</f>
         <v/>
       </c>
       <c r="J95" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J85,ordens_de_servico!I85,"")</f>
+        <f>IF($D$5=ordens_de_servico!J89,ordens_de_servico!I89,"")</f>
         <v/>
       </c>
     </row>
     <row r="96" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F96" s="7" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G96" s="8" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="H96" s="9">
-        <v>46314</v>
+        <v>46322</v>
       </c>
       <c r="I96" s="10" t="str">
-        <f>IF(ordens_de_servico!H86&gt;ordens_de_servico!G86,-DATEDIF(ordens_de_servico!G86,ordens_de_servico!H86,"d"),IF(ordens_de_servico!H86=0,"",DATEDIF(ordens_de_servico!H86,ordens_de_servico!G86,"d")))</f>
+        <f>IF(ordens_de_servico!H90&gt;ordens_de_servico!G90,-DATEDIF(ordens_de_servico!G90,ordens_de_servico!H90,"d"),IF(ordens_de_servico!H90=0,"",DATEDIF(ordens_de_servico!H90,ordens_de_servico!G90,"d")))</f>
         <v/>
       </c>
       <c r="J96" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J86,ordens_de_servico!I86,"")</f>
+        <f>IF($D$5=ordens_de_servico!J90,ordens_de_servico!I90,"")</f>
         <v/>
       </c>
     </row>
     <row r="97" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F97" s="7" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G97" s="8" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="H97" s="9">
-        <v>46315</v>
+        <v>46319</v>
       </c>
       <c r="I97" s="10" t="str">
-        <f>IF(ordens_de_servico!H87&gt;ordens_de_servico!G87,-DATEDIF(ordens_de_servico!G87,ordens_de_servico!H87,"d"),IF(ordens_de_servico!H87=0,"",DATEDIF(ordens_de_servico!H87,ordens_de_servico!G87,"d")))</f>
+        <f>IF(ordens_de_servico!H91&gt;ordens_de_servico!G91,-DATEDIF(ordens_de_servico!G91,ordens_de_servico!H91,"d"),IF(ordens_de_servico!H91=0,"",DATEDIF(ordens_de_servico!H91,ordens_de_servico!G91,"d")))</f>
         <v/>
       </c>
       <c r="J97" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J87,ordens_de_servico!I87,"")</f>
+        <f>IF($D$5=ordens_de_servico!J91,ordens_de_servico!I91,"")</f>
         <v/>
       </c>
     </row>
     <row r="98" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F98" s="7" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G98" s="8" t="s">
-        <v>40</v>
+        <v>116</v>
       </c>
       <c r="H98" s="9">
-        <v>46325</v>
+        <v>46323</v>
       </c>
       <c r="I98" s="10" t="str">
-        <f>IF(ordens_de_servico!H88&gt;ordens_de_servico!G88,-DATEDIF(ordens_de_servico!G88,ordens_de_servico!H88,"d"),IF(ordens_de_servico!H88=0,"",DATEDIF(ordens_de_servico!H88,ordens_de_servico!G88,"d")))</f>
+        <f>IF(ordens_de_servico!H92&gt;ordens_de_servico!G92,-DATEDIF(ordens_de_servico!G92,ordens_de_servico!H92,"d"),IF(ordens_de_servico!H92=0,"",DATEDIF(ordens_de_servico!H92,ordens_de_servico!G92,"d")))</f>
         <v/>
       </c>
       <c r="J98" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J88,ordens_de_servico!I88,"")</f>
+        <f>IF($D$5=ordens_de_servico!J92,ordens_de_servico!I92,"")</f>
         <v/>
       </c>
     </row>
     <row r="99" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F99" s="7" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="G99" s="8" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="H99" s="9">
-        <v>46317</v>
+        <v>46323</v>
       </c>
       <c r="I99" s="10" t="str">
-        <f>IF(ordens_de_servico!H89&gt;ordens_de_servico!G89,-DATEDIF(ordens_de_servico!G89,ordens_de_servico!H89,"d"),IF(ordens_de_servico!H89=0,"",DATEDIF(ordens_de_servico!H89,ordens_de_servico!G89,"d")))</f>
+        <f>IF(ordens_de_servico!H93&gt;ordens_de_servico!G93,-DATEDIF(ordens_de_servico!G93,ordens_de_servico!H93,"d"),IF(ordens_de_servico!H93=0,"",DATEDIF(ordens_de_servico!H93,ordens_de_servico!G93,"d")))</f>
         <v/>
       </c>
       <c r="J99" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J89,ordens_de_servico!I89,"")</f>
+        <f>IF($D$5=ordens_de_servico!J93,ordens_de_servico!I93,"")</f>
         <v/>
       </c>
     </row>
     <row r="100" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F100" s="7" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="H100" s="9">
-        <v>46322</v>
+        <v>46337</v>
       </c>
       <c r="I100" s="10" t="str">
-        <f>IF(ordens_de_servico!H90&gt;ordens_de_servico!G90,-DATEDIF(ordens_de_servico!G90,ordens_de_servico!H90,"d"),IF(ordens_de_servico!H90=0,"",DATEDIF(ordens_de_servico!H90,ordens_de_servico!G90,"d")))</f>
+        <f>IF(ordens_de_servico!H94&gt;ordens_de_servico!G94,-DATEDIF(ordens_de_servico!G94,ordens_de_servico!H94,"d"),IF(ordens_de_servico!H94=0,"",DATEDIF(ordens_de_servico!H94,ordens_de_servico!G94,"d")))</f>
         <v/>
       </c>
       <c r="J100" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J90,ordens_de_servico!I90,"")</f>
+        <f>IF($D$5=ordens_de_servico!J94,ordens_de_servico!I94,"")</f>
         <v/>
       </c>
     </row>
     <row r="101" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F101" s="7" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="G101" s="8" t="s">
-        <v>11</v>
+        <v>56</v>
       </c>
       <c r="H101" s="9">
-        <v>46319</v>
+        <v>46334</v>
       </c>
       <c r="I101" s="10" t="str">
-        <f>IF(ordens_de_servico!H91&gt;ordens_de_servico!G91,-DATEDIF(ordens_de_servico!G91,ordens_de_servico!H91,"d"),IF(ordens_de_servico!H91=0,"",DATEDIF(ordens_de_servico!H91,ordens_de_servico!G91,"d")))</f>
+        <f>IF(ordens_de_servico!H95&gt;ordens_de_servico!G95,-DATEDIF(ordens_de_servico!G95,ordens_de_servico!H95,"d"),IF(ordens_de_servico!H95=0,"",DATEDIF(ordens_de_servico!H95,ordens_de_servico!G95,"d")))</f>
         <v/>
       </c>
       <c r="J101" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J91,ordens_de_servico!I91,"")</f>
+        <f>IF($D$5=ordens_de_servico!J95,ordens_de_servico!I95,"")</f>
         <v/>
       </c>
     </row>
     <row r="102" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F102" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="G102" s="8" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="H102" s="9">
-        <v>46323</v>
+        <v>46331</v>
       </c>
       <c r="I102" s="10" t="str">
-        <f>IF(ordens_de_servico!H92&gt;ordens_de_servico!G92,-DATEDIF(ordens_de_servico!G92,ordens_de_servico!H92,"d"),IF(ordens_de_servico!H92=0,"",DATEDIF(ordens_de_servico!H92,ordens_de_servico!G92,"d")))</f>
+        <f>IF(ordens_de_servico!H96&gt;ordens_de_servico!G96,-DATEDIF(ordens_de_servico!G96,ordens_de_servico!H96,"d"),IF(ordens_de_servico!H96=0,"",DATEDIF(ordens_de_servico!H96,ordens_de_servico!G96,"d")))</f>
         <v/>
       </c>
       <c r="J102" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J92,ordens_de_servico!I92,"")</f>
+        <f>IF($D$5=ordens_de_servico!J96,ordens_de_servico!I96,"")</f>
         <v/>
       </c>
     </row>
     <row r="103" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F103" s="7" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>19</v>
+        <v>116</v>
       </c>
       <c r="H103" s="9">
-        <v>46323</v>
+        <v>46331</v>
       </c>
       <c r="I103" s="10" t="str">
-        <f>IF(ordens_de_servico!H93&gt;ordens_de_servico!G93,-DATEDIF(ordens_de_servico!G93,ordens_de_servico!H93,"d"),IF(ordens_de_servico!H93=0,"",DATEDIF(ordens_de_servico!H93,ordens_de_servico!G93,"d")))</f>
+        <f>IF(ordens_de_servico!H97&gt;ordens_de_servico!G97,-DATEDIF(ordens_de_servico!G97,ordens_de_servico!H97,"d"),IF(ordens_de_servico!H97=0,"",DATEDIF(ordens_de_servico!H97,ordens_de_servico!G97,"d")))</f>
         <v/>
       </c>
       <c r="J103" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J93,ordens_de_servico!I93,"")</f>
+        <f>IF($D$5=ordens_de_servico!J97,ordens_de_servico!I97,"")</f>
         <v/>
       </c>
     </row>
     <row r="104" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F104" s="7" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="G104" s="8" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H104" s="9">
-        <v>46337</v>
+        <v>46329</v>
       </c>
       <c r="I104" s="10" t="str">
-        <f>IF(ordens_de_servico!H94&gt;ordens_de_servico!G94,-DATEDIF(ordens_de_servico!G94,ordens_de_servico!H94,"d"),IF(ordens_de_servico!H94=0,"",DATEDIF(ordens_de_servico!H94,ordens_de_servico!G94,"d")))</f>
+        <f>IF(ordens_de_servico!H98&gt;ordens_de_servico!G98,-DATEDIF(ordens_de_servico!G98,ordens_de_servico!H98,"d"),IF(ordens_de_servico!H98=0,"",DATEDIF(ordens_de_servico!H98,ordens_de_servico!G98,"d")))</f>
         <v/>
       </c>
       <c r="J104" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J94,ordens_de_servico!I94,"")</f>
+        <f>IF($D$5=ordens_de_servico!J98,ordens_de_servico!I98,"")</f>
         <v/>
       </c>
     </row>
     <row r="105" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F105" s="7" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="G105" s="8" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="H105" s="9">
-        <v>46334</v>
+        <v>46333</v>
       </c>
       <c r="I105" s="10" t="str">
-        <f>IF(ordens_de_servico!H95&gt;ordens_de_servico!G95,-DATEDIF(ordens_de_servico!G95,ordens_de_servico!H95,"d"),IF(ordens_de_servico!H95=0,"",DATEDIF(ordens_de_servico!H95,ordens_de_servico!G95,"d")))</f>
+        <f>IF(ordens_de_servico!H99&gt;ordens_de_servico!G99,-DATEDIF(ordens_de_servico!G99,ordens_de_servico!H99,"d"),IF(ordens_de_servico!H99=0,"",DATEDIF(ordens_de_servico!H99,ordens_de_servico!G99,"d")))</f>
         <v/>
       </c>
       <c r="J105" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J95,ordens_de_servico!I95,"")</f>
+        <f>IF($D$5=ordens_de_servico!J99,ordens_de_servico!I99,"")</f>
         <v/>
       </c>
     </row>
     <row r="106" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F106" s="7" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="G106" s="8" t="s">
-        <v>34</v>
+        <v>108</v>
       </c>
       <c r="H106" s="9">
-        <v>46331</v>
+        <v>46334</v>
       </c>
       <c r="I106" s="10" t="str">
-        <f>IF(ordens_de_servico!H96&gt;ordens_de_servico!G96,-DATEDIF(ordens_de_servico!G96,ordens_de_servico!H96,"d"),IF(ordens_de_servico!H96=0,"",DATEDIF(ordens_de_servico!H96,ordens_de_servico!G96,"d")))</f>
+        <f>IF(ordens_de_servico!H100&gt;ordens_de_servico!G100,-DATEDIF(ordens_de_servico!G100,ordens_de_servico!H100,"d"),IF(ordens_de_servico!H100=0,"",DATEDIF(ordens_de_servico!H100,ordens_de_servico!G100,"d")))</f>
         <v/>
       </c>
       <c r="J106" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J96,ordens_de_servico!I96,"")</f>
+        <f>IF($D$5=ordens_de_servico!J100,ordens_de_servico!I100,"")</f>
         <v/>
       </c>
     </row>
     <row r="107" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F107" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="G107" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="H107" s="9">
-        <v>46331</v>
-      </c>
-      <c r="I107" s="10" t="str">
-        <f>IF(ordens_de_servico!H97&gt;ordens_de_servico!G97,-DATEDIF(ordens_de_servico!G97,ordens_de_servico!H97,"d"),IF(ordens_de_servico!H97=0,"",DATEDIF(ordens_de_servico!H97,ordens_de_servico!G97,"d")))</f>
-        <v/>
-      </c>
-      <c r="J107" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J97,ordens_de_servico!I97,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="108" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F108" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="G108" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="H108" s="9">
-        <v>46329</v>
-      </c>
-      <c r="I108" s="10" t="str">
-        <f>IF(ordens_de_servico!H98&gt;ordens_de_servico!G98,-DATEDIF(ordens_de_servico!G98,ordens_de_servico!H98,"d"),IF(ordens_de_servico!H98=0,"",DATEDIF(ordens_de_servico!H98,ordens_de_servico!G98,"d")))</f>
-        <v/>
-      </c>
-      <c r="J108" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J98,ordens_de_servico!I98,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="109" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F109" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="G109" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="H109" s="9">
-        <v>46333</v>
-      </c>
-      <c r="I109" s="10" t="str">
-        <f>IF(ordens_de_servico!H99&gt;ordens_de_servico!G99,-DATEDIF(ordens_de_servico!G99,ordens_de_servico!H99,"d"),IF(ordens_de_servico!H99=0,"",DATEDIF(ordens_de_servico!H99,ordens_de_servico!G99,"d")))</f>
-        <v/>
-      </c>
-      <c r="J109" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J99,ordens_de_servico!I99,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="110" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F110" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="G110" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H110" s="9">
+      <c r="F107" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G107" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="H107" s="14">
         <v>46334</v>
       </c>
-      <c r="I110" s="10" t="str">
-        <f>IF(ordens_de_servico!H100&gt;ordens_de_servico!G100,-DATEDIF(ordens_de_servico!G100,ordens_de_servico!H100,"d"),IF(ordens_de_servico!H100=0,"",DATEDIF(ordens_de_servico!H100,ordens_de_servico!G100,"d")))</f>
-        <v/>
-      </c>
-      <c r="J110" s="11" t="str">
-        <f>IF($D$9=ordens_de_servico!J100,ordens_de_servico!I100,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111" spans="6:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F111" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="G111" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="H111" s="14">
-        <v>46334</v>
-      </c>
-      <c r="I111" s="15" t="str">
+      <c r="I107" s="15" t="str">
         <f>IF(ordens_de_servico!H101&gt;ordens_de_servico!G101,-DATEDIF(ordens_de_servico!G101,ordens_de_servico!H101,"d"),IF(ordens_de_servico!H101=0,"",DATEDIF(ordens_de_servico!H101,ordens_de_servico!G101,"d")))</f>
         <v/>
       </c>
-      <c r="J111" s="16" t="str">
-        <f>IF($D$9=ordens_de_servico!J101,ordens_de_servico!I101,"")</f>
+      <c r="J107" s="16" t="str">
+        <f>IF($D$5=ordens_de_servico!J101,ordens_de_servico!I101,"")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="F11:J111" xr:uid="{14B8D296-2926-4BF5-8E29-9FB41C0EEE9F}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C17:C22">
-    <sortCondition ref="C17:C22"/>
+  <autoFilter ref="F7:J107" xr:uid="{14B8D296-2926-4BF5-8E29-9FB41C0EEE9F}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C13:C18">
+    <sortCondition ref="C13:C18"/>
   </sortState>
   <mergeCells count="1">
-    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C7:D7"/>
   </mergeCells>
-  <conditionalFormatting sqref="F12:J111">
+  <conditionalFormatting sqref="F8:J107">
     <cfRule type="expression" dxfId="3" priority="5">
-      <formula>$J12="Aberta"</formula>
+      <formula>$J8="Aberta"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="6">
-      <formula>$J12="Em andamento"</formula>
+      <formula>$J8="Em andamento"</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="7">
-      <formula>$J12="Concluída"</formula>
+      <formula>$J8="Concluída"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12:I111">
+  <conditionalFormatting sqref="I8:I107">
     <cfRule type="cellIs" dxfId="0" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations xWindow="472" yWindow="308" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor não permitido" error="Escolha uma das opções da lista. Não é possível digitar outro texto neste campo." promptTitle="Filtro" prompt="Selecione o responsável desejado" sqref="D9" xr:uid="{78BEE481-69E3-40B6-91E7-F4B089E9070C}">
+  <dataValidations xWindow="471" yWindow="365" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor não permitido" error="Escolha uma das opções da lista. Não é possível digitar outro texto neste campo." promptTitle="Filtro" prompt="Selecione o responsável desejado" sqref="D5" xr:uid="{78BEE481-69E3-40B6-91E7-F4B089E9070C}">
       <formula1>"Geral,Ana Souza, Carlos Lima, Juliana Alves, Marcos Pereira, Paula Mendes, Rafael Costa"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>